<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-19 12:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4945" uniqueCount="2581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4944" uniqueCount="2581">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19172,9 +19172,6 @@
       </c>
       <c r="D287" t="s">
         <v>1086</v>
-      </c>
-      <c r="E287" t="s">
-        <v>1271</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-20 00:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4944" uniqueCount="2581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4945" uniqueCount="2581">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19172,6 +19172,9 @@
       </c>
       <c r="D287" t="s">
         <v>1086</v>
+      </c>
+      <c r="E287" t="s">
+        <v>1271</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-20 12:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4945" uniqueCount="2581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4944" uniqueCount="2581">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19172,9 +19172,6 @@
       </c>
       <c r="D287" t="s">
         <v>1086</v>
-      </c>
-      <c r="E287" t="s">
-        <v>1271</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-20 18:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4944" uniqueCount="2581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4945" uniqueCount="2581">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19172,6 +19172,9 @@
       </c>
       <c r="D287" t="s">
         <v>1086</v>
+      </c>
+      <c r="E287" t="s">
+        <v>1271</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-21 00:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4945" uniqueCount="2581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4944" uniqueCount="2581">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19172,9 +19172,6 @@
       </c>
       <c r="D287" t="s">
         <v>1086</v>
-      </c>
-      <c r="E287" t="s">
-        <v>1271</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-23 12:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4944" uniqueCount="2581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4945" uniqueCount="2581">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19172,6 +19172,9 @@
       </c>
       <c r="D287" t="s">
         <v>1086</v>
+      </c>
+      <c r="E287" t="s">
+        <v>1271</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-24 00:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4945" uniqueCount="2581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4944" uniqueCount="2581">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19172,9 +19172,6 @@
       </c>
       <c r="D287" t="s">
         <v>1086</v>
-      </c>
-      <c r="E287" t="s">
-        <v>1271</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-24 18:30:04
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -4087,6 +4087,9 @@
     <t>ORÇAMENTO</t>
   </si>
   <si>
+    <t>BIOLOGIA,URBANISMO</t>
+  </si>
+  <si>
     <t>MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
@@ -4130,9 +4133,6 @@
   </si>
   <si>
     <t>ECONOMICIDADE OBRAS,ENGENHARIA CIVIL</t>
-  </si>
-  <si>
-    <t>BIOLOGIA,URBANISMO</t>
   </si>
   <si>
     <t>EDIFICAÇÕES</t>
@@ -10815,7 +10815,7 @@
         <v>1341</v>
       </c>
       <c r="H36" t="s">
-        <v>1349</v>
+        <v>1357</v>
       </c>
       <c r="I36" t="s">
         <v>1420</v>
@@ -11007,7 +11007,7 @@
         <v>1341</v>
       </c>
       <c r="H42" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="I42" t="s">
         <v>1406</v>
@@ -11141,7 +11141,7 @@
         <v>1341</v>
       </c>
       <c r="H46" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="I46" t="s">
         <v>1405</v>
@@ -11173,7 +11173,7 @@
         <v>1341</v>
       </c>
       <c r="H47" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="I47" t="s">
         <v>1429</v>
@@ -11307,7 +11307,7 @@
         <v>1341</v>
       </c>
       <c r="H51" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="I51" t="s">
         <v>1431</v>
@@ -11371,7 +11371,7 @@
         <v>1344</v>
       </c>
       <c r="H53" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="I53" t="s">
         <v>1433</v>
@@ -11601,7 +11601,7 @@
         <v>1343</v>
       </c>
       <c r="H60" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="I60" t="s">
         <v>1438</v>
@@ -11633,7 +11633,7 @@
         <v>1341</v>
       </c>
       <c r="H61" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I61" t="s">
         <v>1423</v>
@@ -11700,7 +11700,7 @@
         <v>1341</v>
       </c>
       <c r="H63" t="s">
-        <v>1363</v>
+        <v>1364</v>
       </c>
       <c r="I63" t="s">
         <v>1396</v>
@@ -11959,7 +11959,7 @@
         <v>1341</v>
       </c>
       <c r="H71" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I71" t="s">
         <v>1442</v>
@@ -11994,7 +11994,7 @@
         <v>1341</v>
       </c>
       <c r="H72" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I72" t="s">
         <v>1443</v>
@@ -12026,7 +12026,7 @@
         <v>1342</v>
       </c>
       <c r="H73" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
       <c r="I73" t="s">
         <v>1429</v>
@@ -12396,7 +12396,7 @@
         <v>1341</v>
       </c>
       <c r="H84" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I84" t="s">
         <v>1442</v>
@@ -12463,7 +12463,7 @@
         <v>1341</v>
       </c>
       <c r="H86" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I86" t="s">
         <v>1449</v>
@@ -12530,7 +12530,7 @@
         <v>1341</v>
       </c>
       <c r="H88" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I88" t="s">
         <v>1442</v>
@@ -12603,7 +12603,7 @@
         <v>1343</v>
       </c>
       <c r="H90" t="s">
-        <v>1366</v>
+        <v>1367</v>
       </c>
       <c r="I90" t="s">
         <v>1403</v>
@@ -12903,7 +12903,7 @@
         <v>1341</v>
       </c>
       <c r="H99" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I99" t="s">
         <v>1442</v>
@@ -13101,7 +13101,7 @@
         <v>1341</v>
       </c>
       <c r="H105" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="I105" t="s">
         <v>1453</v>
@@ -13343,7 +13343,7 @@
         <v>1341</v>
       </c>
       <c r="H112" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="I112" t="s">
         <v>1458</v>
@@ -13471,7 +13471,7 @@
         <v>1341</v>
       </c>
       <c r="H116" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="I116" t="s">
         <v>1460</v>
@@ -13503,7 +13503,7 @@
         <v>1341</v>
       </c>
       <c r="H117" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="I117" t="s">
         <v>1397</v>
@@ -13701,7 +13701,7 @@
         <v>1341</v>
       </c>
       <c r="H123" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I123" t="s">
         <v>1462</v>
@@ -13733,7 +13733,7 @@
         <v>1341</v>
       </c>
       <c r="H124" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
       <c r="I124" t="s">
         <v>1403</v>
@@ -13829,7 +13829,7 @@
         <v>1341</v>
       </c>
       <c r="H127" t="s">
-        <v>1371</v>
+        <v>1372</v>
       </c>
       <c r="I127" t="s">
         <v>1441</v>
@@ -13861,7 +13861,7 @@
         <v>1342</v>
       </c>
       <c r="H128" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="I128" t="s">
         <v>1463</v>
@@ -13989,7 +13989,7 @@
         <v>1341</v>
       </c>
       <c r="H132" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I132" t="s">
         <v>1423</v>
@@ -14085,7 +14085,7 @@
         <v>1341</v>
       </c>
       <c r="H135" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="I135" t="s">
         <v>1465</v>
@@ -14219,7 +14219,7 @@
         <v>1341</v>
       </c>
       <c r="H139" t="s">
-        <v>1370</v>
+        <v>1371</v>
       </c>
       <c r="I139" t="s">
         <v>1420</v>
@@ -14353,7 +14353,7 @@
         <v>1342</v>
       </c>
       <c r="H143" t="s">
-        <v>1372</v>
+        <v>1357</v>
       </c>
       <c r="I143" t="s">
         <v>1397</v>
@@ -14455,7 +14455,7 @@
         <v>1341</v>
       </c>
       <c r="H146" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I146" t="s">
         <v>1460</v>
@@ -14630,7 +14630,7 @@
         <v>1343</v>
       </c>
       <c r="H151" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="I151" t="s">
         <v>1473</v>
@@ -14697,7 +14697,7 @@
         <v>1341</v>
       </c>
       <c r="H153" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I153" t="s">
         <v>1471</v>
@@ -14863,7 +14863,7 @@
         <v>1341</v>
       </c>
       <c r="H158" t="s">
-        <v>1365</v>
+        <v>1366</v>
       </c>
       <c r="I158" t="s">
         <v>1476</v>
@@ -15000,7 +15000,7 @@
         <v>1341</v>
       </c>
       <c r="H162" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="I162" t="s">
         <v>1478</v>
@@ -15064,7 +15064,7 @@
         <v>1341</v>
       </c>
       <c r="H164" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I164" t="s">
         <v>1409</v>
@@ -15254,7 +15254,7 @@
         <v>1341</v>
       </c>
       <c r="H169" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="I169" t="s">
         <v>1427</v>
@@ -15330,7 +15330,7 @@
         <v>1341</v>
       </c>
       <c r="H171" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="I171" t="s">
         <v>1397</v>
@@ -15726,7 +15726,7 @@
         <v>1341</v>
       </c>
       <c r="H183" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="I183" t="s">
         <v>1465</v>
@@ -15962,7 +15962,7 @@
         <v>1342</v>
       </c>
       <c r="H190" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="I190" t="s">
         <v>1478</v>
@@ -16419,7 +16419,7 @@
         <v>1341</v>
       </c>
       <c r="H204" t="s">
-        <v>1372</v>
+        <v>1357</v>
       </c>
       <c r="I204" t="s">
         <v>1438</v>
@@ -16661,7 +16661,7 @@
         <v>1342</v>
       </c>
       <c r="H211" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="I211" t="s">
         <v>1400</v>
@@ -17159,7 +17159,7 @@
         <v>1342</v>
       </c>
       <c r="H226" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I226" t="s">
         <v>1494</v>
@@ -18091,7 +18091,7 @@
         <v>1341</v>
       </c>
       <c r="H254" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I254" t="s">
         <v>1483</v>
@@ -18123,7 +18123,7 @@
         <v>1342</v>
       </c>
       <c r="H255" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="I255" t="s">
         <v>1466</v>
@@ -18193,7 +18193,7 @@
         <v>1341</v>
       </c>
       <c r="H257" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="I257" t="s">
         <v>1451</v>
@@ -19672,7 +19672,7 @@
         <v>1341</v>
       </c>
       <c r="H302" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="I302" t="s">
         <v>1481</v>
@@ -19748,7 +19748,7 @@
         <v>1341</v>
       </c>
       <c r="H304" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I304" t="s">
         <v>1507</v>
@@ -20141,7 +20141,7 @@
         <v>1341</v>
       </c>
       <c r="H316" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I316" t="s">
         <v>1471</v>
@@ -20307,7 +20307,7 @@
         <v>1341</v>
       </c>
       <c r="H321" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I321" t="s">
         <v>1442</v>
@@ -20473,7 +20473,7 @@
         <v>1341</v>
       </c>
       <c r="H326" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I326" t="s">
         <v>1449</v>
@@ -20639,7 +20639,7 @@
         <v>1341</v>
       </c>
       <c r="H331" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I331" t="s">
         <v>1442</v>
@@ -21096,7 +21096,7 @@
         <v>1341</v>
       </c>
       <c r="H345" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="I345" t="s">
         <v>1449</v>
@@ -21553,7 +21553,7 @@
         <v>1341</v>
       </c>
       <c r="H359" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="I359" t="s">
         <v>1396</v>
@@ -21591,7 +21591,7 @@
         <v>1341</v>
       </c>
       <c r="H360" t="s">
-        <v>1369</v>
+        <v>1370</v>
       </c>
       <c r="I360" t="s">
         <v>1397</v>
@@ -21655,7 +21655,7 @@
         <v>1341</v>
       </c>
       <c r="H362" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I362" t="s">
         <v>1447</v>
@@ -21859,7 +21859,7 @@
         <v>1341</v>
       </c>
       <c r="H368" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="I368" t="s">
         <v>1516</v>
@@ -22098,7 +22098,7 @@
         <v>1341</v>
       </c>
       <c r="H375" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I375" t="s">
         <v>1519</v>
@@ -22459,7 +22459,7 @@
         <v>1341</v>
       </c>
       <c r="H386" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I386" t="s">
         <v>1485</v>
@@ -22491,7 +22491,7 @@
         <v>1341</v>
       </c>
       <c r="H387" t="s">
-        <v>1361</v>
+        <v>1362</v>
       </c>
       <c r="I387" t="s">
         <v>1431</v>
@@ -22692,7 +22692,7 @@
         <v>1341</v>
       </c>
       <c r="H393" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I393" t="s">
         <v>1449</v>
@@ -22788,7 +22788,7 @@
         <v>1342</v>
       </c>
       <c r="H396" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="I396" t="s">
         <v>1400</v>
@@ -22858,7 +22858,7 @@
         <v>1343</v>
       </c>
       <c r="H398" t="s">
-        <v>1367</v>
+        <v>1368</v>
       </c>
       <c r="I398" t="s">
         <v>1473</v>
@@ -23100,7 +23100,7 @@
         <v>1341</v>
       </c>
       <c r="H405" t="s">
-        <v>1357</v>
+        <v>1358</v>
       </c>
       <c r="I405" t="s">
         <v>1427</v>
@@ -23365,7 +23365,7 @@
         <v>1341</v>
       </c>
       <c r="H413" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I413" t="s">
         <v>1523</v>
@@ -23633,7 +23633,7 @@
         <v>1341</v>
       </c>
       <c r="H421" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I421" t="s">
         <v>1449</v>
@@ -24839,7 +24839,7 @@
         <v>1341</v>
       </c>
       <c r="H457" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I457" t="s">
         <v>1483</v>
@@ -25343,7 +25343,7 @@
         <v>1341</v>
       </c>
       <c r="H472" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I472" t="s">
         <v>1471</v>
@@ -25375,7 +25375,7 @@
         <v>1341</v>
       </c>
       <c r="H473" t="s">
-        <v>1359</v>
+        <v>1360</v>
       </c>
       <c r="I473" t="s">
         <v>1433</v>
@@ -25506,7 +25506,7 @@
         <v>1341</v>
       </c>
       <c r="H477" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I477" t="s">
         <v>1396</v>
@@ -25538,7 +25538,7 @@
         <v>1342</v>
       </c>
       <c r="H478" t="s">
-        <v>1360</v>
+        <v>1361</v>
       </c>
       <c r="I478" t="s">
         <v>1396</v>
@@ -25602,7 +25602,7 @@
         <v>1341</v>
       </c>
       <c r="H480" t="s">
-        <v>1362</v>
+        <v>1363</v>
       </c>
       <c r="I480" t="s">
         <v>1519</v>
@@ -25771,7 +25771,7 @@
         <v>1341</v>
       </c>
       <c r="H485" t="s">
-        <v>1364</v>
+        <v>1365</v>
       </c>
       <c r="I485" t="s">
         <v>1471</v>
@@ -26252,7 +26252,7 @@
         <v>1341</v>
       </c>
       <c r="H499" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="I499" t="s">
         <v>1427</v>
@@ -26686,7 +26686,7 @@
         <v>1341</v>
       </c>
       <c r="H512" t="s">
-        <v>1358</v>
+        <v>1359</v>
       </c>
       <c r="I512" t="s">
         <v>1438</v>
@@ -27085,7 +27085,7 @@
         <v>1341</v>
       </c>
       <c r="H524" t="s">
-        <v>1368</v>
+        <v>1369</v>
       </c>
       <c r="I524" t="s">
         <v>1427</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-25 12:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4944" uniqueCount="2581">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4945" uniqueCount="2581">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19172,6 +19172,9 @@
       </c>
       <c r="D287" t="s">
         <v>1086</v>
+      </c>
+      <c r="E287" t="s">
+        <v>1271</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-26 18:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4927" uniqueCount="2573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4926" uniqueCount="2573">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19116,9 +19116,6 @@
       </c>
       <c r="D286" t="s">
         <v>1082</v>
-      </c>
-      <c r="E286" t="s">
-        <v>1267</v>
       </c>
       <c r="F286" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-27 00:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4926" uniqueCount="2573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4927" uniqueCount="2573">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19117,6 +19117,9 @@
       <c r="D286" t="s">
         <v>1082</v>
       </c>
+      <c r="E286" t="s">
+        <v>1267</v>
+      </c>
       <c r="F286" s="2">
         <v>45771</v>
       </c>
@@ -20277,7 +20280,7 @@
         <v>1163</v>
       </c>
       <c r="F321" s="2">
-        <v>45708</v>
+        <v>46079</v>
       </c>
       <c r="G321" t="s">
         <v>1337</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-02-27 12:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4927" uniqueCount="2573">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4926" uniqueCount="2573">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19116,9 +19116,6 @@
       </c>
       <c r="D286" t="s">
         <v>1082</v>
-      </c>
-      <c r="E286" t="s">
-        <v>1267</v>
       </c>
       <c r="F286" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-03 18:30:04
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4919" uniqueCount="2571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4920" uniqueCount="2571">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19135,6 +19135,9 @@
       </c>
       <c r="D287" t="s">
         <v>1080</v>
+      </c>
+      <c r="E287" t="s">
+        <v>1266</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-04 00:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4920" uniqueCount="2571">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4919" uniqueCount="2571">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19135,9 +19135,6 @@
       </c>
       <c r="D287" t="s">
         <v>1080</v>
-      </c>
-      <c r="E287" t="s">
-        <v>1266</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-05 00:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4910" uniqueCount="2567">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4911" uniqueCount="2567">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19114,6 +19114,9 @@
       </c>
       <c r="D287" t="s">
         <v>1078</v>
+      </c>
+      <c r="E287" t="s">
+        <v>1264</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-05 12:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4911" uniqueCount="2567">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4910" uniqueCount="2567">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19114,9 +19114,6 @@
       </c>
       <c r="D287" t="s">
         <v>1078</v>
-      </c>
-      <c r="E287" t="s">
-        <v>1264</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-06 12:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4910" uniqueCount="2567">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4911" uniqueCount="2567">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -19114,6 +19114,9 @@
       </c>
       <c r="D287" t="s">
         <v>1078</v>
+      </c>
+      <c r="E287" t="s">
+        <v>1264</v>
       </c>
       <c r="F287" s="2">
         <v>45771</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-03-16 14:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -4636,6 +4636,9 @@
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO</t>
   </si>
   <si>
+    <t>AVALIAÇÃO DE IMÓVEIS</t>
+  </si>
+  <si>
     <t>FENOMENOS DE ENERGIA E INFORMAÇÃO,MOBILIDADE E TRANSPORTE</t>
   </si>
   <si>
@@ -4709,9 +4712,6 @@
   </si>
   <si>
     <t>MOBILIDADE E TRANSPORTE,VALORAÇÃO DANOS AMBIENTAIS</t>
-  </si>
-  <si>
-    <t>AVALIAÇÃO DE IMÓVEIS</t>
   </si>
   <si>
     <t>BIOLOGIA,GEOLOGIA</t>
@@ -13215,7 +13215,7 @@
         <v>1525</v>
       </c>
       <c r="H69" t="s">
-        <v>1529</v>
+        <v>1540</v>
       </c>
       <c r="I69" t="s">
         <v>1627</v>
@@ -13413,7 +13413,7 @@
         <v>1528</v>
       </c>
       <c r="H75" t="s">
-        <v>1540</v>
+        <v>1541</v>
       </c>
       <c r="I75" t="s">
         <v>1632</v>
@@ -14042,7 +14042,7 @@
         <v>1525</v>
       </c>
       <c r="H94" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="I94" t="s">
         <v>1640</v>
@@ -14246,7 +14246,7 @@
         <v>1525</v>
       </c>
       <c r="H100" t="s">
-        <v>1542</v>
+        <v>1543</v>
       </c>
       <c r="I100" t="s">
         <v>1612</v>
@@ -14278,7 +14278,7 @@
         <v>1525</v>
       </c>
       <c r="H101" t="s">
-        <v>1543</v>
+        <v>1544</v>
       </c>
       <c r="I101" t="s">
         <v>1636</v>
@@ -14552,7 +14552,7 @@
         <v>1525</v>
       </c>
       <c r="H109" t="s">
-        <v>1544</v>
+        <v>1545</v>
       </c>
       <c r="I109" t="s">
         <v>1580</v>
@@ -14756,7 +14756,7 @@
         <v>1525</v>
       </c>
       <c r="H115" t="s">
-        <v>1545</v>
+        <v>1546</v>
       </c>
       <c r="I115" t="s">
         <v>1609</v>
@@ -15379,7 +15379,7 @@
         <v>1525</v>
       </c>
       <c r="H134" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
       <c r="I134" t="s">
         <v>1653</v>
@@ -15417,7 +15417,7 @@
         <v>1525</v>
       </c>
       <c r="H135" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
       <c r="I135" t="s">
         <v>1632</v>
@@ -15493,7 +15493,7 @@
         <v>1525</v>
       </c>
       <c r="H137" t="s">
-        <v>1547</v>
+        <v>1548</v>
       </c>
       <c r="I137" t="s">
         <v>1654</v>
@@ -15621,7 +15621,7 @@
         <v>1525</v>
       </c>
       <c r="H141" t="s">
-        <v>1548</v>
+        <v>1549</v>
       </c>
       <c r="I141" t="s">
         <v>1656</v>
@@ -15723,7 +15723,7 @@
         <v>1525</v>
       </c>
       <c r="H144" t="s">
-        <v>1549</v>
+        <v>1550</v>
       </c>
       <c r="I144" t="s">
         <v>1606</v>
@@ -15915,7 +15915,7 @@
         <v>1525</v>
       </c>
       <c r="H150" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="I150" t="s">
         <v>1657</v>
@@ -15947,7 +15947,7 @@
         <v>1525</v>
       </c>
       <c r="H151" t="s">
-        <v>1551</v>
+        <v>1552</v>
       </c>
       <c r="I151" t="s">
         <v>1585</v>
@@ -16468,7 +16468,7 @@
         <v>1525</v>
       </c>
       <c r="H167" t="s">
-        <v>1552</v>
+        <v>1553</v>
       </c>
       <c r="I167" t="s">
         <v>1606</v>
@@ -16666,7 +16666,7 @@
         <v>1526</v>
       </c>
       <c r="H173" t="s">
-        <v>1553</v>
+        <v>1554</v>
       </c>
       <c r="I173" t="s">
         <v>1578</v>
@@ -16768,7 +16768,7 @@
         <v>1525</v>
       </c>
       <c r="H176" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="I176" t="s">
         <v>1656</v>
@@ -17473,7 +17473,7 @@
         <v>1525</v>
       </c>
       <c r="H197" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="I197" t="s">
         <v>1593</v>
@@ -17549,7 +17549,7 @@
         <v>1525</v>
       </c>
       <c r="H199" t="s">
-        <v>1554</v>
+        <v>1555</v>
       </c>
       <c r="I199" t="s">
         <v>1674</v>
@@ -18467,7 +18467,7 @@
         <v>1525</v>
       </c>
       <c r="H226" t="s">
-        <v>1542</v>
+        <v>1543</v>
       </c>
       <c r="I226" t="s">
         <v>1681</v>
@@ -19172,7 +19172,7 @@
         <v>1526</v>
       </c>
       <c r="H247" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
       <c r="I247" t="s">
         <v>1686</v>
@@ -19405,7 +19405,7 @@
         <v>1525</v>
       </c>
       <c r="H254" t="s">
-        <v>1551</v>
+        <v>1552</v>
       </c>
       <c r="I254" t="s">
         <v>1615</v>
@@ -19638,7 +19638,7 @@
         <v>1525</v>
       </c>
       <c r="H261" t="s">
-        <v>1555</v>
+        <v>1556</v>
       </c>
       <c r="I261" t="s">
         <v>1671</v>
@@ -19708,7 +19708,7 @@
         <v>1525</v>
       </c>
       <c r="H263" t="s">
-        <v>1556</v>
+        <v>1557</v>
       </c>
       <c r="I263" t="s">
         <v>1633</v>
@@ -19804,7 +19804,7 @@
         <v>1527</v>
       </c>
       <c r="H266" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
       <c r="I266" t="s">
         <v>1591</v>
@@ -20215,7 +20215,7 @@
         <v>1525</v>
       </c>
       <c r="H278" t="s">
-        <v>1558</v>
+        <v>1559</v>
       </c>
       <c r="I278" t="s">
         <v>1620</v>
@@ -20736,7 +20736,7 @@
         <v>1525</v>
       </c>
       <c r="H294" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
       <c r="I294" t="s">
         <v>1581</v>
@@ -20806,7 +20806,7 @@
         <v>1525</v>
       </c>
       <c r="H296" t="s">
-        <v>1560</v>
+        <v>1561</v>
       </c>
       <c r="I296" t="s">
         <v>1678</v>
@@ -21170,7 +21170,7 @@
         <v>1526</v>
       </c>
       <c r="H307" t="s">
-        <v>1561</v>
+        <v>1562</v>
       </c>
       <c r="I307" t="s">
         <v>1592</v>
@@ -21828,7 +21828,7 @@
         <v>1525</v>
       </c>
       <c r="H327" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="I327" t="s">
         <v>1581</v>
@@ -21866,7 +21866,7 @@
         <v>1525</v>
       </c>
       <c r="H328" t="s">
-        <v>1562</v>
+        <v>1563</v>
       </c>
       <c r="I328" t="s">
         <v>1699</v>
@@ -22198,7 +22198,7 @@
         <v>1525</v>
       </c>
       <c r="H338" t="s">
-        <v>1563</v>
+        <v>1564</v>
       </c>
       <c r="I338" t="s">
         <v>1701</v>
@@ -22332,7 +22332,7 @@
         <v>1525</v>
       </c>
       <c r="H342" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
       <c r="I342" t="s">
         <v>1661</v>
@@ -22504,7 +22504,7 @@
         <v>1525</v>
       </c>
       <c r="H347" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="I347" t="s">
         <v>1703</v>
@@ -22862,7 +22862,7 @@
         <v>1525</v>
       </c>
       <c r="H358" t="s">
-        <v>1564</v>
+        <v>1565</v>
       </c>
       <c r="I358" t="s">
         <v>1632</v>
@@ -23124,7 +23124,7 @@
         <v>1525</v>
       </c>
       <c r="H366" t="s">
-        <v>1565</v>
+        <v>1540</v>
       </c>
       <c r="I366" t="s">
         <v>1615</v>
@@ -23357,7 +23357,7 @@
         <v>1525</v>
       </c>
       <c r="H373" t="s">
-        <v>1543</v>
+        <v>1544</v>
       </c>
       <c r="I373" t="s">
         <v>1614</v>
@@ -23555,7 +23555,7 @@
         <v>1525</v>
       </c>
       <c r="H379" t="s">
-        <v>1543</v>
+        <v>1544</v>
       </c>
       <c r="I379" t="s">
         <v>1636</v>
@@ -23654,7 +23654,7 @@
         <v>1525</v>
       </c>
       <c r="H382" t="s">
-        <v>1544</v>
+        <v>1545</v>
       </c>
       <c r="I382" t="s">
         <v>1707</v>
@@ -24006,7 +24006,7 @@
         <v>1525</v>
       </c>
       <c r="H393" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="I393" t="s">
         <v>1702</v>
@@ -24335,7 +24335,7 @@
         <v>1525</v>
       </c>
       <c r="H403" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
       <c r="I403" t="s">
         <v>1713</v>
@@ -25206,7 +25206,7 @@
         <v>1525</v>
       </c>
       <c r="H429" t="s">
-        <v>1545</v>
+        <v>1546</v>
       </c>
       <c r="I429" t="s">
         <v>1678</v>
@@ -25244,7 +25244,7 @@
         <v>1525</v>
       </c>
       <c r="H430" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="I430" t="s">
         <v>1691</v>
@@ -25509,7 +25509,7 @@
         <v>1525</v>
       </c>
       <c r="H438" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
       <c r="I438" t="s">
         <v>1659</v>
@@ -26042,7 +26042,7 @@
         <v>1525</v>
       </c>
       <c r="H454" t="s">
-        <v>1565</v>
+        <v>1540</v>
       </c>
       <c r="I454" t="s">
         <v>1656</v>
@@ -26619,7 +26619,7 @@
         <v>1525</v>
       </c>
       <c r="H471" t="s">
-        <v>1554</v>
+        <v>1555</v>
       </c>
       <c r="I471" t="s">
         <v>1645</v>
@@ -27254,7 +27254,7 @@
         <v>1527</v>
       </c>
       <c r="H490" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
       <c r="I490" t="s">
         <v>1723</v>
@@ -27554,7 +27554,7 @@
         <v>1525</v>
       </c>
       <c r="H499" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="I499" t="s">
         <v>1689</v>
@@ -27918,7 +27918,7 @@
         <v>1525</v>
       </c>
       <c r="H510" t="s">
-        <v>1544</v>
+        <v>1545</v>
       </c>
       <c r="I510" t="s">
         <v>1685</v>
@@ -28256,7 +28256,7 @@
         <v>1525</v>
       </c>
       <c r="H520" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="I520" t="s">
         <v>1678</v>
@@ -28632,7 +28632,7 @@
         <v>1525</v>
       </c>
       <c r="H531" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
       <c r="I531" t="s">
         <v>1713</v>
@@ -29057,7 +29057,7 @@
         <v>1525</v>
       </c>
       <c r="H544" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="I544" t="s">
         <v>1691</v>
@@ -29541,7 +29541,7 @@
         <v>1528</v>
       </c>
       <c r="H558" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="I558" t="s">
         <v>1581</v>
@@ -30109,7 +30109,7 @@
         <v>1525</v>
       </c>
       <c r="H575" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
       <c r="I575" t="s">
         <v>1585</v>
@@ -30415,7 +30415,7 @@
         <v>1528</v>
       </c>
       <c r="H584" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="I584" t="s">
         <v>1623</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-04-14 10:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -12681,7 +12681,7 @@
         <v>45908</v>
       </c>
       <c r="G34" t="s">
-        <v>1606</v>
+        <v>1608</v>
       </c>
       <c r="H34" t="s">
         <v>1612</v>
@@ -13953,7 +13953,7 @@
         <v>45994</v>
       </c>
       <c r="G73" t="s">
-        <v>1608</v>
+        <v>1606</v>
       </c>
       <c r="H73" t="s">
         <v>1631</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-04-27 12:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -4924,6 +4924,9 @@
     <t>###   SEM TEMA   ###</t>
   </si>
   <si>
+    <t>MEDICINA LEGAL</t>
+  </si>
+  <si>
     <t>URBANISMO</t>
   </si>
   <si>
@@ -4931,9 +4934,6 @@
   </si>
   <si>
     <t>FARMÁCIA,SAÚDE</t>
-  </si>
-  <si>
-    <t>MEDICINA LEGAL</t>
   </si>
   <si>
     <t>PATRIMÔNIO HISTÓRICO E CULTURAL</t>
@@ -12020,7 +12020,7 @@
         <v>1627</v>
       </c>
       <c r="H10" t="s">
-        <v>1635</v>
+        <v>1636</v>
       </c>
       <c r="I10" t="s">
         <v>1692</v>
@@ -12058,7 +12058,7 @@
         <v>1630</v>
       </c>
       <c r="H11" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="I11" t="s">
         <v>1693</v>
@@ -12186,7 +12186,7 @@
         <v>1628</v>
       </c>
       <c r="H15" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="I15" t="s">
         <v>1695</v>
@@ -12288,7 +12288,7 @@
         <v>1627</v>
       </c>
       <c r="H18" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="I18" t="s">
         <v>1698</v>
@@ -12326,7 +12326,7 @@
         <v>1627</v>
       </c>
       <c r="H19" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I19" t="s">
         <v>1699</v>
@@ -12524,7 +12524,7 @@
         <v>1627</v>
       </c>
       <c r="H25" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I25" t="s">
         <v>1705</v>
@@ -12559,7 +12559,7 @@
         <v>1627</v>
       </c>
       <c r="H26" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I26" t="s">
         <v>1706</v>
@@ -14355,7 +14355,7 @@
         <v>1627</v>
       </c>
       <c r="H81" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I81" t="s">
         <v>1744</v>
@@ -15363,7 +15363,7 @@
         <v>1627</v>
       </c>
       <c r="H111" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I111" t="s">
         <v>1756</v>
@@ -15640,7 +15640,7 @@
         <v>1628</v>
       </c>
       <c r="H119" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="I119" t="s">
         <v>1710</v>
@@ -15879,7 +15879,7 @@
         <v>1627</v>
       </c>
       <c r="H126" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I126" t="s">
         <v>1760</v>
@@ -16109,7 +16109,7 @@
         <v>1629</v>
       </c>
       <c r="H133" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I133" t="s">
         <v>1762</v>
@@ -16505,7 +16505,7 @@
         <v>1627</v>
       </c>
       <c r="H145" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="I145" t="s">
         <v>1766</v>
@@ -16543,7 +16543,7 @@
         <v>1627</v>
       </c>
       <c r="H146" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="I146" t="s">
         <v>1745</v>
@@ -17789,7 +17789,7 @@
         <v>1627</v>
       </c>
       <c r="H184" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I184" t="s">
         <v>1775</v>
@@ -19127,7 +19127,7 @@
         <v>1627</v>
       </c>
       <c r="H223" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I223" t="s">
         <v>1790</v>
@@ -19488,7 +19488,7 @@
         <v>1629</v>
       </c>
       <c r="H234" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I234" t="s">
         <v>1698</v>
@@ -20400,7 +20400,7 @@
         <v>1628</v>
       </c>
       <c r="H261" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="I261" t="s">
         <v>1799</v>
@@ -20930,7 +20930,7 @@
         <v>1627</v>
       </c>
       <c r="H277" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I277" t="s">
         <v>1804</v>
@@ -21303,7 +21303,7 @@
         <v>1627</v>
       </c>
       <c r="H288" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I288" t="s">
         <v>1734</v>
@@ -21990,7 +21990,7 @@
         <v>1627</v>
       </c>
       <c r="H309" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I309" t="s">
         <v>1810</v>
@@ -22200,7 +22200,7 @@
         <v>1627</v>
       </c>
       <c r="H315" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="I315" t="s">
         <v>1698</v>
@@ -22334,7 +22334,7 @@
         <v>1627</v>
       </c>
       <c r="H319" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I319" t="s">
         <v>1734</v>
@@ -23936,7 +23936,7 @@
         <v>1627</v>
       </c>
       <c r="H367" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="I367" t="s">
         <v>1773</v>
@@ -25153,7 +25153,7 @@
         <v>1627</v>
       </c>
       <c r="H404" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I404" t="s">
         <v>1822</v>
@@ -26976,7 +26976,7 @@
         <v>1627</v>
       </c>
       <c r="H459" t="s">
-        <v>1638</v>
+        <v>1639</v>
       </c>
       <c r="I459" t="s">
         <v>1698</v>
@@ -27509,7 +27509,7 @@
         <v>1627</v>
       </c>
       <c r="H475" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I475" t="s">
         <v>1691</v>
@@ -28086,7 +28086,7 @@
         <v>1627</v>
       </c>
       <c r="H492" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I492" t="s">
         <v>1712</v>
@@ -28928,7 +28928,7 @@
         <v>1627</v>
       </c>
       <c r="H517" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I517" t="s">
         <v>1805</v>
@@ -29583,7 +29583,7 @@
         <v>1627</v>
       </c>
       <c r="H537" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="I537" t="s">
         <v>1738</v>
@@ -30396,7 +30396,7 @@
         <v>1627</v>
       </c>
       <c r="H561" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I561" t="s">
         <v>1839</v>
@@ -31016,7 +31016,7 @@
         <v>1628</v>
       </c>
       <c r="H580" t="s">
-        <v>1637</v>
+        <v>1638</v>
       </c>
       <c r="I580" t="s">
         <v>1695</v>
@@ -31226,7 +31226,7 @@
         <v>1627</v>
       </c>
       <c r="H586" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I586" t="s">
         <v>1717</v>
@@ -32126,7 +32126,7 @@
         <v>1627</v>
       </c>
       <c r="H613" t="s">
-        <v>1636</v>
+        <v>1637</v>
       </c>
       <c r="I613" t="s">
         <v>1693</v>
@@ -32298,7 +32298,7 @@
         <v>1628</v>
       </c>
       <c r="H618" t="s">
-        <v>1639</v>
+        <v>1636</v>
       </c>
       <c r="I618" t="s">
         <v>1842</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-05-12 18:30:04
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -4546,6 +4546,9 @@
     <t>19/03/2026</t>
   </si>
   <si>
+    <t>27/04/2026</t>
+  </si>
+  <si>
     <t>03/09/2025</t>
   </si>
   <si>
@@ -4690,7 +4693,7 @@
     <t>15/06/2025</t>
   </si>
   <si>
-    <t>07/11/2025</t>
+    <t>06/05/2026</t>
   </si>
   <si>
     <t>16/04/2025</t>
@@ -4784,9 +4787,6 @@
   </si>
   <si>
     <t>21/11/2024</t>
-  </si>
-  <si>
-    <t>06/05/2026</t>
   </si>
   <si>
     <t>21/10/2024</t>
@@ -12297,7 +12297,7 @@
         <v>1354</v>
       </c>
       <c r="E11" t="s">
-        <v>1563</v>
+        <v>1564</v>
       </c>
       <c r="F11" s="2">
         <v>45922</v>
@@ -12524,7 +12524,7 @@
         <v>1329</v>
       </c>
       <c r="D18" t="s">
-        <v>1537</v>
+        <v>1538</v>
       </c>
       <c r="E18" t="s">
         <v>1653</v>
@@ -12667,7 +12667,7 @@
         <v>1608</v>
       </c>
       <c r="E22" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="F22" s="2">
         <v>46125</v>
@@ -12798,7 +12798,7 @@
         <v>1337</v>
       </c>
       <c r="D26" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="F26" s="2">
         <v>45889</v>
@@ -13997,7 +13997,7 @@
         <v>1441</v>
       </c>
       <c r="E63" t="s">
-        <v>1567</v>
+        <v>1568</v>
       </c>
       <c r="F63" s="2">
         <v>46112</v>
@@ -14661,10 +14661,10 @@
         <v>1385</v>
       </c>
       <c r="D83" t="s">
-        <v>1517</v>
+        <v>1518</v>
       </c>
       <c r="E83" t="s">
-        <v>1517</v>
+        <v>1518</v>
       </c>
       <c r="F83" s="2">
         <v>45690</v>
@@ -15124,7 +15124,7 @@
         <v>1393</v>
       </c>
       <c r="D97" t="s">
-        <v>1525</v>
+        <v>1526</v>
       </c>
       <c r="F97" s="2">
         <v>45972</v>
@@ -15599,10 +15599,10 @@
         <v>1401</v>
       </c>
       <c r="D111" t="s">
-        <v>1553</v>
+        <v>1554</v>
       </c>
       <c r="E111" t="s">
-        <v>1553</v>
+        <v>1554</v>
       </c>
       <c r="F111" s="2">
         <v>46113</v>
@@ -15637,7 +15637,7 @@
         <v>1402</v>
       </c>
       <c r="D112" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="F112" s="2">
         <v>46009</v>
@@ -15876,10 +15876,10 @@
         <v>1405</v>
       </c>
       <c r="D119" t="s">
-        <v>1548</v>
+        <v>1549</v>
       </c>
       <c r="E119" t="s">
-        <v>1548</v>
+        <v>1549</v>
       </c>
       <c r="F119" s="2">
         <v>46127</v>
@@ -16080,7 +16080,7 @@
         <v>1411</v>
       </c>
       <c r="D125" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="E125" t="s">
         <v>1656</v>
@@ -16386,7 +16386,7 @@
         <v>1414</v>
       </c>
       <c r="E134" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
       <c r="F134" s="2">
         <v>45727</v>
@@ -16590,7 +16590,7 @@
         <v>1608</v>
       </c>
       <c r="E140" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="F140" s="2">
         <v>46126</v>
@@ -17900,7 +17900,7 @@
         <v>1444</v>
       </c>
       <c r="D180" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="E180" t="s">
         <v>1606</v>
@@ -18541,7 +18541,7 @@
         <v>1356</v>
       </c>
       <c r="D199" t="s">
-        <v>1528</v>
+        <v>1529</v>
       </c>
       <c r="F199" s="2">
         <v>45972</v>
@@ -18905,10 +18905,10 @@
         <v>1434</v>
       </c>
       <c r="D210" t="s">
-        <v>1535</v>
+        <v>1536</v>
       </c>
       <c r="E210" t="s">
-        <v>1535</v>
+        <v>1536</v>
       </c>
       <c r="F210" s="2">
         <v>45869</v>
@@ -19220,7 +19220,7 @@
         <v>1622</v>
       </c>
       <c r="E219" t="s">
-        <v>1570</v>
+        <v>1571</v>
       </c>
       <c r="F219" s="2">
         <v>45838</v>
@@ -19296,7 +19296,7 @@
         <v>1623</v>
       </c>
       <c r="E221" t="s">
-        <v>1524</v>
+        <v>1525</v>
       </c>
       <c r="F221" s="2">
         <v>46009</v>
@@ -20059,10 +20059,10 @@
         <v>1480</v>
       </c>
       <c r="D244" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
       <c r="E244" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
       <c r="F244" s="2">
         <v>45860</v>
@@ -21399,7 +21399,7 @@
         <v>1393</v>
       </c>
       <c r="E284" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
       <c r="F284" s="2">
         <v>45919</v>
@@ -21804,7 +21804,7 @@
         <v>1631</v>
       </c>
       <c r="E296" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="F296" s="2">
         <v>45952</v>
@@ -21874,7 +21874,7 @@
         <v>1632</v>
       </c>
       <c r="E298" t="s">
-        <v>1544</v>
+        <v>1545</v>
       </c>
       <c r="F298" s="2">
         <v>45818</v>
@@ -22040,10 +22040,10 @@
         <v>964</v>
       </c>
       <c r="C303" t="s">
-        <v>1316</v>
+        <v>1510</v>
       </c>
       <c r="F303" s="2">
-        <v>45994</v>
+        <v>46154</v>
       </c>
       <c r="G303" t="s">
         <v>1666</v>
@@ -22104,7 +22104,7 @@
         <v>966</v>
       </c>
       <c r="C305" t="s">
-        <v>1510</v>
+        <v>1511</v>
       </c>
       <c r="F305" s="2">
         <v>45994</v>
@@ -22136,7 +22136,7 @@
         <v>967</v>
       </c>
       <c r="C306" t="s">
-        <v>1511</v>
+        <v>1512</v>
       </c>
       <c r="F306" s="2">
         <v>46044</v>
@@ -22203,7 +22203,7 @@
         <v>969</v>
       </c>
       <c r="C308" t="s">
-        <v>1512</v>
+        <v>1513</v>
       </c>
       <c r="F308" s="2">
         <v>45965</v>
@@ -22363,7 +22363,7 @@
         <v>974</v>
       </c>
       <c r="C313" t="s">
-        <v>1513</v>
+        <v>1514</v>
       </c>
       <c r="F313" s="2">
         <v>46118</v>
@@ -22459,7 +22459,7 @@
         <v>977</v>
       </c>
       <c r="C316" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
       <c r="F316" s="2">
         <v>45754</v>
@@ -22491,7 +22491,7 @@
         <v>978</v>
       </c>
       <c r="C317" t="s">
-        <v>1515</v>
+        <v>1516</v>
       </c>
       <c r="F317" s="2">
         <v>46050</v>
@@ -22593,7 +22593,7 @@
         <v>981</v>
       </c>
       <c r="C320" t="s">
-        <v>1516</v>
+        <v>1517</v>
       </c>
       <c r="F320" s="2">
         <v>45883</v>
@@ -22625,7 +22625,7 @@
         <v>982</v>
       </c>
       <c r="C321" t="s">
-        <v>1517</v>
+        <v>1518</v>
       </c>
       <c r="D321" t="s">
         <v>1451</v>
@@ -22663,7 +22663,7 @@
         <v>983</v>
       </c>
       <c r="C322" t="s">
-        <v>1518</v>
+        <v>1519</v>
       </c>
       <c r="F322" s="2">
         <v>46043</v>
@@ -22698,10 +22698,10 @@
         <v>1378</v>
       </c>
       <c r="D323" t="s">
-        <v>1549</v>
+        <v>1550</v>
       </c>
       <c r="E323" t="s">
-        <v>1549</v>
+        <v>1550</v>
       </c>
       <c r="F323" s="2">
         <v>45937</v>
@@ -22733,7 +22733,7 @@
         <v>985</v>
       </c>
       <c r="C324" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
       <c r="F324" s="2">
         <v>45887</v>
@@ -22765,7 +22765,7 @@
         <v>986</v>
       </c>
       <c r="C325" t="s">
-        <v>1520</v>
+        <v>1521</v>
       </c>
       <c r="D325" t="s">
         <v>1636</v>
@@ -22835,7 +22835,7 @@
         <v>988</v>
       </c>
       <c r="C327" t="s">
-        <v>1521</v>
+        <v>1522</v>
       </c>
       <c r="F327" s="2">
         <v>46129</v>
@@ -22899,7 +22899,7 @@
         <v>990</v>
       </c>
       <c r="C329" t="s">
-        <v>1522</v>
+        <v>1523</v>
       </c>
       <c r="F329" s="2">
         <v>46149</v>
@@ -22963,7 +22963,7 @@
         <v>992</v>
       </c>
       <c r="C331" t="s">
-        <v>1523</v>
+        <v>1524</v>
       </c>
       <c r="F331" s="2">
         <v>45799</v>
@@ -22995,7 +22995,7 @@
         <v>993</v>
       </c>
       <c r="C332" t="s">
-        <v>1524</v>
+        <v>1525</v>
       </c>
       <c r="F332" s="2">
         <v>46118</v>
@@ -23155,13 +23155,13 @@
         <v>998</v>
       </c>
       <c r="C337" t="s">
-        <v>1525</v>
+        <v>1526</v>
       </c>
       <c r="D337" t="s">
-        <v>1554</v>
+        <v>1555</v>
       </c>
       <c r="E337" t="s">
-        <v>1554</v>
+        <v>1555</v>
       </c>
       <c r="F337" s="2">
         <v>45972</v>
@@ -23193,7 +23193,7 @@
         <v>999</v>
       </c>
       <c r="C338" t="s">
-        <v>1526</v>
+        <v>1527</v>
       </c>
       <c r="D338" t="s">
         <v>1637</v>
@@ -23231,7 +23231,7 @@
         <v>1000</v>
       </c>
       <c r="C339" t="s">
-        <v>1527</v>
+        <v>1528</v>
       </c>
       <c r="F339" s="2">
         <v>45680</v>
@@ -23263,7 +23263,7 @@
         <v>1001</v>
       </c>
       <c r="C340" t="s">
-        <v>1523</v>
+        <v>1524</v>
       </c>
       <c r="D340" t="s">
         <v>1353</v>
@@ -23333,7 +23333,7 @@
         <v>1003</v>
       </c>
       <c r="C342" t="s">
-        <v>1528</v>
+        <v>1529</v>
       </c>
       <c r="F342" s="2">
         <v>46149</v>
@@ -23365,7 +23365,7 @@
         <v>1004</v>
       </c>
       <c r="C343" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
       <c r="F343" s="2">
         <v>45818</v>
@@ -23429,13 +23429,13 @@
         <v>1006</v>
       </c>
       <c r="C345" t="s">
-        <v>1529</v>
+        <v>1530</v>
       </c>
       <c r="D345" t="s">
         <v>1608</v>
       </c>
       <c r="E345" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="F345" s="2">
         <v>46112</v>
@@ -23563,7 +23563,7 @@
         <v>1010</v>
       </c>
       <c r="C349" t="s">
-        <v>1530</v>
+        <v>1531</v>
       </c>
       <c r="F349" s="2">
         <v>46010</v>
@@ -23595,7 +23595,7 @@
         <v>1011</v>
       </c>
       <c r="C350" t="s">
-        <v>1528</v>
+        <v>1529</v>
       </c>
       <c r="F350" s="2">
         <v>46149</v>
@@ -23627,7 +23627,7 @@
         <v>1012</v>
       </c>
       <c r="C351" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
       <c r="F351" s="2">
         <v>45812</v>
@@ -23691,7 +23691,7 @@
         <v>1014</v>
       </c>
       <c r="C353" t="s">
-        <v>1532</v>
+        <v>1533</v>
       </c>
       <c r="F353" s="2">
         <v>45811</v>
@@ -23755,7 +23755,7 @@
         <v>1016</v>
       </c>
       <c r="C355" t="s">
-        <v>1533</v>
+        <v>1534</v>
       </c>
       <c r="F355" s="2">
         <v>45883</v>
@@ -23787,7 +23787,7 @@
         <v>1017</v>
       </c>
       <c r="C356" t="s">
-        <v>1534</v>
+        <v>1535</v>
       </c>
       <c r="F356" s="2">
         <v>45846</v>
@@ -23883,7 +23883,7 @@
         <v>1020</v>
       </c>
       <c r="C359" t="s">
-        <v>1535</v>
+        <v>1536</v>
       </c>
       <c r="F359" s="2">
         <v>45870</v>
@@ -23915,7 +23915,7 @@
         <v>1021</v>
       </c>
       <c r="C360" t="s">
-        <v>1536</v>
+        <v>1537</v>
       </c>
       <c r="F360" s="2">
         <v>45751</v>
@@ -23947,7 +23947,7 @@
         <v>1022</v>
       </c>
       <c r="C361" t="s">
-        <v>1537</v>
+        <v>1538</v>
       </c>
       <c r="D361" t="s">
         <v>1638</v>
@@ -24029,7 +24029,7 @@
         <v>1350</v>
       </c>
       <c r="E363" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
       <c r="F363" s="2">
         <v>45771</v>
@@ -24093,7 +24093,7 @@
         <v>1026</v>
       </c>
       <c r="C365" t="s">
-        <v>1538</v>
+        <v>1539</v>
       </c>
       <c r="F365" s="2">
         <v>45728</v>
@@ -24157,13 +24157,13 @@
         <v>1028</v>
       </c>
       <c r="C367" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="D367" t="s">
         <v>1639</v>
       </c>
       <c r="E367" t="s">
-        <v>1568</v>
+        <v>1569</v>
       </c>
       <c r="F367" s="2">
         <v>46139</v>
@@ -24259,7 +24259,7 @@
         <v>1031</v>
       </c>
       <c r="C370" t="s">
-        <v>1540</v>
+        <v>1541</v>
       </c>
       <c r="F370" s="2">
         <v>46092</v>
@@ -24294,10 +24294,10 @@
         <v>1457</v>
       </c>
       <c r="D371" t="s">
-        <v>1529</v>
+        <v>1530</v>
       </c>
       <c r="E371" t="s">
-        <v>1529</v>
+        <v>1530</v>
       </c>
       <c r="F371" s="2">
         <v>46091</v>
@@ -24329,7 +24329,7 @@
         <v>1033</v>
       </c>
       <c r="C372" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="F372" s="2">
         <v>46035</v>
@@ -24399,7 +24399,7 @@
         <v>1035</v>
       </c>
       <c r="C374" t="s">
-        <v>1542</v>
+        <v>1543</v>
       </c>
       <c r="F374" s="2">
         <v>45659</v>
@@ -24431,7 +24431,7 @@
         <v>1036</v>
       </c>
       <c r="C375" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
       <c r="F375" s="2">
         <v>45891</v>
@@ -24495,7 +24495,7 @@
         <v>1038</v>
       </c>
       <c r="C377" t="s">
-        <v>1543</v>
+        <v>1544</v>
       </c>
       <c r="F377" s="2">
         <v>45728</v>
@@ -24527,7 +24527,7 @@
         <v>1039</v>
       </c>
       <c r="C378" t="s">
-        <v>1544</v>
+        <v>1545</v>
       </c>
       <c r="D378" t="s">
         <v>1338</v>
@@ -24629,7 +24629,7 @@
         <v>1042</v>
       </c>
       <c r="C381" t="s">
-        <v>1545</v>
+        <v>1546</v>
       </c>
       <c r="F381" s="2">
         <v>46048</v>
@@ -24664,7 +24664,7 @@
         <v>1391</v>
       </c>
       <c r="D382" t="s">
-        <v>1534</v>
+        <v>1535</v>
       </c>
       <c r="E382" t="s">
         <v>1403</v>
@@ -24737,7 +24737,7 @@
         <v>1045</v>
       </c>
       <c r="C384" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
       <c r="F384" s="2">
         <v>46044</v>
@@ -24769,7 +24769,7 @@
         <v>1046</v>
       </c>
       <c r="C385" t="s">
-        <v>1547</v>
+        <v>1548</v>
       </c>
       <c r="F385" s="2">
         <v>45868</v>
@@ -24833,7 +24833,7 @@
         <v>1048</v>
       </c>
       <c r="C387" t="s">
-        <v>1548</v>
+        <v>1549</v>
       </c>
       <c r="F387" s="2">
         <v>46149</v>
@@ -24929,7 +24929,7 @@
         <v>1051</v>
       </c>
       <c r="C390" t="s">
-        <v>1549</v>
+        <v>1550</v>
       </c>
       <c r="F390" s="2">
         <v>46092</v>
@@ -25057,7 +25057,7 @@
         <v>1055</v>
       </c>
       <c r="C394" t="s">
-        <v>1522</v>
+        <v>1523</v>
       </c>
       <c r="F394" s="2">
         <v>46149</v>
@@ -25121,7 +25121,7 @@
         <v>1057</v>
       </c>
       <c r="C396" t="s">
-        <v>1550</v>
+        <v>1551</v>
       </c>
       <c r="D396" t="s">
         <v>1641</v>
@@ -25159,7 +25159,7 @@
         <v>1058</v>
       </c>
       <c r="C397" t="s">
-        <v>1551</v>
+        <v>1552</v>
       </c>
       <c r="F397" s="2">
         <v>45877</v>
@@ -25191,7 +25191,7 @@
         <v>1059</v>
       </c>
       <c r="C398" t="s">
-        <v>1552</v>
+        <v>1553</v>
       </c>
       <c r="D398" t="s">
         <v>1642</v>
@@ -25226,7 +25226,7 @@
         <v>1060</v>
       </c>
       <c r="C399" t="s">
-        <v>1553</v>
+        <v>1554</v>
       </c>
       <c r="F399" s="2">
         <v>46118</v>
@@ -25290,7 +25290,7 @@
         <v>1062</v>
       </c>
       <c r="C401" t="s">
-        <v>1554</v>
+        <v>1555</v>
       </c>
       <c r="F401" s="2">
         <v>45993</v>
@@ -25389,7 +25389,7 @@
         <v>1065</v>
       </c>
       <c r="C404" t="s">
-        <v>1555</v>
+        <v>1556</v>
       </c>
       <c r="F404" s="2">
         <v>46120</v>
@@ -25421,7 +25421,7 @@
         <v>1066</v>
       </c>
       <c r="C405" t="s">
-        <v>1556</v>
+        <v>1557</v>
       </c>
       <c r="D405" t="s">
         <v>1643</v>
@@ -25488,7 +25488,7 @@
         <v>1068</v>
       </c>
       <c r="C407" t="s">
-        <v>1551</v>
+        <v>1552</v>
       </c>
       <c r="F407" s="2">
         <v>45853</v>
@@ -25552,7 +25552,7 @@
         <v>1070</v>
       </c>
       <c r="C409" t="s">
-        <v>1557</v>
+        <v>1558</v>
       </c>
       <c r="F409" s="2">
         <v>45852</v>
@@ -25651,7 +25651,7 @@
         <v>1073</v>
       </c>
       <c r="C412" t="s">
-        <v>1516</v>
+        <v>1517</v>
       </c>
       <c r="F412" s="2">
         <v>46035</v>
@@ -25683,10 +25683,10 @@
         <v>1074</v>
       </c>
       <c r="C413" t="s">
-        <v>1558</v>
+        <v>1559</v>
       </c>
       <c r="F413" s="2">
-        <v>46044</v>
+        <v>46154</v>
       </c>
       <c r="G413" t="s">
         <v>1666</v>
@@ -25753,7 +25753,7 @@
         <v>1076</v>
       </c>
       <c r="C415" t="s">
-        <v>1534</v>
+        <v>1535</v>
       </c>
       <c r="F415" s="2">
         <v>45946</v>
@@ -25913,7 +25913,7 @@
         <v>1081</v>
       </c>
       <c r="C420" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
       <c r="D420" t="s">
         <v>1644</v>
@@ -25951,7 +25951,7 @@
         <v>1082</v>
       </c>
       <c r="C421" t="s">
-        <v>1559</v>
+        <v>1560</v>
       </c>
       <c r="F421" s="2">
         <v>45825</v>
@@ -26018,7 +26018,7 @@
         <v>1320</v>
       </c>
       <c r="D423" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="F423" s="2">
         <v>45952</v>
@@ -26242,7 +26242,7 @@
         <v>1091</v>
       </c>
       <c r="C430" t="s">
-        <v>1513</v>
+        <v>1514</v>
       </c>
       <c r="F430" s="2">
         <v>46112</v>
@@ -26274,7 +26274,7 @@
         <v>1092</v>
       </c>
       <c r="C431" t="s">
-        <v>1560</v>
+        <v>1561</v>
       </c>
       <c r="F431" s="2">
         <v>45680</v>
@@ -26370,7 +26370,7 @@
         <v>1095</v>
       </c>
       <c r="C434" t="s">
-        <v>1533</v>
+        <v>1534</v>
       </c>
       <c r="F434" s="2">
         <v>45714</v>
@@ -26402,7 +26402,7 @@
         <v>1096</v>
       </c>
       <c r="C435" t="s">
-        <v>1561</v>
+        <v>1562</v>
       </c>
       <c r="F435" s="2">
         <v>45671</v>
@@ -26504,7 +26504,7 @@
         <v>1415</v>
       </c>
       <c r="E438" t="s">
-        <v>1571</v>
+        <v>1572</v>
       </c>
       <c r="F438" s="2">
         <v>45929</v>
@@ -26536,7 +26536,7 @@
         <v>1100</v>
       </c>
       <c r="C439" t="s">
-        <v>1562</v>
+        <v>1563</v>
       </c>
       <c r="F439" s="2">
         <v>45799</v>
@@ -26699,7 +26699,7 @@
         <v>1427</v>
       </c>
       <c r="D444" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
       <c r="F444" s="2">
         <v>45812</v>
@@ -26763,7 +26763,7 @@
         <v>1107</v>
       </c>
       <c r="C446" t="s">
-        <v>1563</v>
+        <v>1564</v>
       </c>
       <c r="F446" s="2">
         <v>45994</v>
@@ -26859,7 +26859,7 @@
         <v>1110</v>
       </c>
       <c r="C449" t="s">
-        <v>1564</v>
+        <v>1565</v>
       </c>
       <c r="F449" s="2">
         <v>45673</v>
@@ -26891,7 +26891,7 @@
         <v>1111</v>
       </c>
       <c r="C450" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
       <c r="F450" s="2">
         <v>45919</v>
@@ -27019,7 +27019,7 @@
         <v>1115</v>
       </c>
       <c r="C454" t="s">
-        <v>1566</v>
+        <v>1567</v>
       </c>
       <c r="D454" t="s">
         <v>1470</v>
@@ -27095,7 +27095,7 @@
         <v>1117</v>
       </c>
       <c r="C456" t="s">
-        <v>1567</v>
+        <v>1568</v>
       </c>
       <c r="F456" s="2">
         <v>45989</v>
@@ -27127,7 +27127,7 @@
         <v>1118</v>
       </c>
       <c r="C457" t="s">
-        <v>1568</v>
+        <v>1569</v>
       </c>
       <c r="D457" t="s">
         <v>1639</v>
@@ -27200,7 +27200,7 @@
         <v>1363</v>
       </c>
       <c r="E459" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="F459" s="2">
         <v>45924</v>
@@ -27296,7 +27296,7 @@
         <v>1123</v>
       </c>
       <c r="C462" t="s">
-        <v>1569</v>
+        <v>1570</v>
       </c>
       <c r="D462" t="s">
         <v>1488</v>
@@ -27337,7 +27337,7 @@
         <v>1394</v>
       </c>
       <c r="D463" t="s">
-        <v>1510</v>
+        <v>1511</v>
       </c>
       <c r="E463" t="s">
         <v>1347</v>
@@ -27404,7 +27404,7 @@
         <v>1126</v>
       </c>
       <c r="C465" t="s">
-        <v>1527</v>
+        <v>1528</v>
       </c>
       <c r="F465" s="2">
         <v>45693</v>
@@ -27436,7 +27436,7 @@
         <v>1127</v>
       </c>
       <c r="C466" t="s">
-        <v>1570</v>
+        <v>1571</v>
       </c>
       <c r="F466" s="2">
         <v>45735</v>
@@ -27468,7 +27468,7 @@
         <v>1128</v>
       </c>
       <c r="C467" t="s">
-        <v>1571</v>
+        <v>1572</v>
       </c>
       <c r="F467" s="2">
         <v>46028</v>
@@ -27503,10 +27503,10 @@
         <v>1339</v>
       </c>
       <c r="D468" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="E468" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="F468" s="2">
         <v>46118</v>
@@ -27538,7 +27538,7 @@
         <v>1130</v>
       </c>
       <c r="C469" t="s">
-        <v>1532</v>
+        <v>1533</v>
       </c>
       <c r="F469" s="2">
         <v>45812</v>
@@ -27605,7 +27605,7 @@
         <v>1132</v>
       </c>
       <c r="C471" t="s">
-        <v>1549</v>
+        <v>1550</v>
       </c>
       <c r="F471" s="2">
         <v>46148</v>
@@ -27637,7 +27637,7 @@
         <v>1133</v>
       </c>
       <c r="C472" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
       <c r="F472" s="2">
         <v>46044</v>
@@ -27742,10 +27742,10 @@
         <v>1428</v>
       </c>
       <c r="D475" t="s">
-        <v>1532</v>
+        <v>1533</v>
       </c>
       <c r="E475" t="s">
-        <v>1532</v>
+        <v>1533</v>
       </c>
       <c r="F475" s="2">
         <v>45811</v>
@@ -27777,7 +27777,7 @@
         <v>1137</v>
       </c>
       <c r="C476" t="s">
-        <v>1532</v>
+        <v>1533</v>
       </c>
       <c r="F476" s="2">
         <v>45897</v>
@@ -27841,7 +27841,7 @@
         <v>1139</v>
       </c>
       <c r="C478" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
       <c r="F478" s="2">
         <v>45754</v>
@@ -27905,7 +27905,7 @@
         <v>1141</v>
       </c>
       <c r="C480" t="s">
-        <v>1533</v>
+        <v>1534</v>
       </c>
       <c r="D480" t="s">
         <v>1645</v>
@@ -28042,7 +28042,7 @@
         <v>1145</v>
       </c>
       <c r="C484" t="s">
-        <v>1565</v>
+        <v>1566</v>
       </c>
       <c r="F484" s="2">
         <v>45995</v>
@@ -28240,7 +28240,7 @@
         <v>1621</v>
       </c>
       <c r="E490" t="s">
-        <v>1524</v>
+        <v>1525</v>
       </c>
       <c r="F490" s="2">
         <v>45992</v>
@@ -28272,7 +28272,7 @@
         <v>1152</v>
       </c>
       <c r="C491" t="s">
-        <v>1572</v>
+        <v>1573</v>
       </c>
       <c r="F491" s="2">
         <v>46010</v>
@@ -28304,7 +28304,7 @@
         <v>1153</v>
       </c>
       <c r="C492" t="s">
-        <v>1573</v>
+        <v>1574</v>
       </c>
       <c r="D492" t="s">
         <v>1392</v>
@@ -28339,7 +28339,7 @@
         <v>1154</v>
       </c>
       <c r="C493" t="s">
-        <v>1566</v>
+        <v>1567</v>
       </c>
       <c r="F493" s="2">
         <v>45849</v>
@@ -28435,7 +28435,7 @@
         <v>1157</v>
       </c>
       <c r="C496" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="F496" s="2">
         <v>45811</v>
@@ -28543,7 +28543,7 @@
         <v>1160</v>
       </c>
       <c r="C499" t="s">
-        <v>1575</v>
+        <v>1576</v>
       </c>
       <c r="F499" s="2">
         <v>45684</v>
@@ -28575,7 +28575,7 @@
         <v>1161</v>
       </c>
       <c r="C500" t="s">
-        <v>1576</v>
+        <v>1577</v>
       </c>
       <c r="F500" s="2">
         <v>46092</v>
@@ -28607,7 +28607,7 @@
         <v>1162</v>
       </c>
       <c r="C501" t="s">
-        <v>1577</v>
+        <v>1578</v>
       </c>
       <c r="D501" t="s">
         <v>1647</v>
@@ -28782,7 +28782,7 @@
         <v>1344</v>
       </c>
       <c r="D506" t="s">
-        <v>1566</v>
+        <v>1567</v>
       </c>
       <c r="E506" t="s">
         <v>1477</v>
@@ -28817,7 +28817,7 @@
         <v>1168</v>
       </c>
       <c r="C507" t="s">
-        <v>1574</v>
+        <v>1575</v>
       </c>
       <c r="F507" s="2">
         <v>45722</v>
@@ -28945,7 +28945,7 @@
         <v>1172</v>
       </c>
       <c r="C511" t="s">
-        <v>1547</v>
+        <v>1548</v>
       </c>
       <c r="F511" s="2">
         <v>45994</v>
@@ -29012,7 +29012,7 @@
         <v>1174</v>
       </c>
       <c r="C513" t="s">
-        <v>1578</v>
+        <v>1579</v>
       </c>
       <c r="D513" t="s">
         <v>1478</v>
@@ -29050,7 +29050,7 @@
         <v>1175</v>
       </c>
       <c r="C514" t="s">
-        <v>1579</v>
+        <v>1580</v>
       </c>
       <c r="F514" s="2">
         <v>45679</v>
@@ -29085,10 +29085,10 @@
         <v>1448</v>
       </c>
       <c r="D515" t="s">
-        <v>1542</v>
+        <v>1543</v>
       </c>
       <c r="E515" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="F515" s="2">
         <v>45915</v>
@@ -29420,7 +29420,7 @@
         <v>1186</v>
       </c>
       <c r="C525" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="F525" s="2">
         <v>45824</v>
@@ -29519,7 +29519,7 @@
         <v>1189</v>
       </c>
       <c r="C528" t="s">
-        <v>1547</v>
+        <v>1548</v>
       </c>
       <c r="F528" s="2">
         <v>46093</v>
@@ -29551,13 +29551,13 @@
         <v>1190</v>
       </c>
       <c r="C529" t="s">
-        <v>1543</v>
+        <v>1544</v>
       </c>
       <c r="D529" t="s">
         <v>1473</v>
       </c>
       <c r="E529" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
       <c r="F529" s="2">
         <v>45750</v>
@@ -29621,7 +29621,7 @@
         <v>1192</v>
       </c>
       <c r="C531" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="F531" s="2">
         <v>45946</v>
@@ -29653,7 +29653,7 @@
         <v>1193</v>
       </c>
       <c r="C532" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="F532" s="2">
         <v>45751</v>
@@ -29781,7 +29781,7 @@
         <v>1197</v>
       </c>
       <c r="C536" t="s">
-        <v>1516</v>
+        <v>1517</v>
       </c>
       <c r="F536" s="2">
         <v>45994</v>
@@ -29851,7 +29851,7 @@
         <v>1199</v>
       </c>
       <c r="C538" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="F538" s="2">
         <v>46049</v>
@@ -29979,7 +29979,7 @@
         <v>1203</v>
       </c>
       <c r="C542" t="s">
-        <v>1583</v>
+        <v>1584</v>
       </c>
       <c r="F542" s="2">
         <v>45722</v>
@@ -30011,7 +30011,7 @@
         <v>1204</v>
       </c>
       <c r="C543" t="s">
-        <v>1584</v>
+        <v>1585</v>
       </c>
       <c r="F543" s="2">
         <v>45994</v>
@@ -30043,7 +30043,7 @@
         <v>1205</v>
       </c>
       <c r="C544" t="s">
-        <v>1585</v>
+        <v>1586</v>
       </c>
       <c r="D544" t="s">
         <v>1405</v>
@@ -30081,7 +30081,7 @@
         <v>1206</v>
       </c>
       <c r="C545" t="s">
-        <v>1586</v>
+        <v>1587</v>
       </c>
       <c r="F545" s="2">
         <v>46127</v>
@@ -30113,7 +30113,7 @@
         <v>1207</v>
       </c>
       <c r="C546" t="s">
-        <v>1536</v>
+        <v>1537</v>
       </c>
       <c r="F546" s="2">
         <v>45730</v>
@@ -30148,7 +30148,7 @@
         <v>1376</v>
       </c>
       <c r="D547" t="s">
-        <v>1579</v>
+        <v>1580</v>
       </c>
       <c r="F547" s="2">
         <v>45709</v>
@@ -30404,7 +30404,7 @@
         <v>1216</v>
       </c>
       <c r="C555" t="s">
-        <v>1587</v>
+        <v>1588</v>
       </c>
       <c r="D555" t="s">
         <v>1649</v>
@@ -30503,7 +30503,7 @@
         <v>1219</v>
       </c>
       <c r="C558" t="s">
-        <v>1588</v>
+        <v>1589</v>
       </c>
       <c r="D558" t="s">
         <v>1650</v>
@@ -30541,7 +30541,7 @@
         <v>1220</v>
       </c>
       <c r="C559" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="F559" s="2">
         <v>45751</v>
@@ -30637,7 +30637,7 @@
         <v>1223</v>
       </c>
       <c r="C562" t="s">
-        <v>1589</v>
+        <v>1590</v>
       </c>
       <c r="F562" s="2">
         <v>45684</v>
@@ -30733,7 +30733,7 @@
         <v>1226</v>
       </c>
       <c r="C565" t="s">
-        <v>1590</v>
+        <v>1559</v>
       </c>
       <c r="F565" s="2">
         <v>46150</v>
@@ -30978,10 +30978,10 @@
         <v>1448</v>
       </c>
       <c r="D572" t="s">
-        <v>1531</v>
+        <v>1532</v>
       </c>
       <c r="E572" t="s">
-        <v>1546</v>
+        <v>1547</v>
       </c>
       <c r="F572" s="2">
         <v>45992</v>
@@ -31115,7 +31115,7 @@
         <v>1237</v>
       </c>
       <c r="C576" t="s">
-        <v>1533</v>
+        <v>1534</v>
       </c>
       <c r="F576" s="2">
         <v>45751</v>
@@ -31153,7 +31153,7 @@
         <v>1623</v>
       </c>
       <c r="E577" t="s">
-        <v>1580</v>
+        <v>1581</v>
       </c>
       <c r="F577" s="2">
         <v>45946</v>
@@ -31185,7 +31185,7 @@
         <v>1239</v>
       </c>
       <c r="C578" t="s">
-        <v>1572</v>
+        <v>1573</v>
       </c>
       <c r="F578" s="2">
         <v>45888</v>
@@ -31281,13 +31281,13 @@
         <v>1242</v>
       </c>
       <c r="C581" t="s">
-        <v>1573</v>
+        <v>1574</v>
       </c>
       <c r="D581" t="s">
         <v>1507</v>
       </c>
       <c r="E581" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="F581" s="2">
         <v>45894</v>
@@ -31319,7 +31319,7 @@
         <v>1243</v>
       </c>
       <c r="C582" t="s">
-        <v>1530</v>
+        <v>1531</v>
       </c>
       <c r="F582" s="2">
         <v>46010</v>
@@ -31450,7 +31450,7 @@
         <v>1247</v>
       </c>
       <c r="C586" t="s">
-        <v>1537</v>
+        <v>1538</v>
       </c>
       <c r="F586" s="2">
         <v>46112</v>
@@ -31482,7 +31482,7 @@
         <v>1248</v>
       </c>
       <c r="C587" t="s">
-        <v>1570</v>
+        <v>1571</v>
       </c>
       <c r="F587" s="2">
         <v>45735</v>
@@ -31546,7 +31546,7 @@
         <v>1250</v>
       </c>
       <c r="C589" t="s">
-        <v>1560</v>
+        <v>1561</v>
       </c>
       <c r="F589" s="2">
         <v>45715</v>
@@ -31980,7 +31980,7 @@
         <v>1350</v>
       </c>
       <c r="D602" t="s">
-        <v>1538</v>
+        <v>1539</v>
       </c>
       <c r="F602" s="2">
         <v>45870</v>
@@ -32076,7 +32076,7 @@
         <v>1266</v>
       </c>
       <c r="C605" t="s">
-        <v>1545</v>
+        <v>1546</v>
       </c>
       <c r="F605" s="2">
         <v>46118</v>
@@ -32175,10 +32175,10 @@
         <v>1598</v>
       </c>
       <c r="D608" t="s">
-        <v>1578</v>
+        <v>1579</v>
       </c>
       <c r="E608" t="s">
-        <v>1578</v>
+        <v>1579</v>
       </c>
       <c r="F608" s="2">
         <v>45946</v>
@@ -32216,7 +32216,7 @@
         <v>1349</v>
       </c>
       <c r="E609" t="s">
-        <v>1582</v>
+        <v>1583</v>
       </c>
       <c r="F609" s="2">
         <v>45975</v>
@@ -32280,7 +32280,7 @@
         <v>1272</v>
       </c>
       <c r="C611" t="s">
-        <v>1524</v>
+        <v>1525</v>
       </c>
       <c r="F611" s="2">
         <v>46092</v>
@@ -32350,7 +32350,7 @@
         <v>1358</v>
       </c>
       <c r="E613" t="s">
-        <v>1581</v>
+        <v>1582</v>
       </c>
       <c r="F613" s="2">
         <v>45704</v>
@@ -32516,7 +32516,7 @@
         <v>1279</v>
       </c>
       <c r="C618" t="s">
-        <v>1560</v>
+        <v>1561</v>
       </c>
       <c r="F618" s="2">
         <v>45811</v>
@@ -32586,7 +32586,7 @@
         <v>1391</v>
       </c>
       <c r="E620" t="s">
-        <v>1519</v>
+        <v>1520</v>
       </c>
       <c r="F620" s="2">
         <v>46045</v>
@@ -32650,7 +32650,7 @@
         <v>1283</v>
       </c>
       <c r="C622" t="s">
-        <v>1528</v>
+        <v>1529</v>
       </c>
       <c r="F622" s="2">
         <v>45925</v>
@@ -32714,7 +32714,7 @@
         <v>1285</v>
       </c>
       <c r="C624" t="s">
-        <v>1548</v>
+        <v>1549</v>
       </c>
       <c r="F624" s="2">
         <v>46091</v>
@@ -32810,7 +32810,7 @@
         <v>1288</v>
       </c>
       <c r="C627" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="F627" s="2">
         <v>46118</v>
@@ -33256,7 +33256,7 @@
         <v>1325</v>
       </c>
       <c r="E640" t="s">
-        <v>1539</v>
+        <v>1540</v>
       </c>
       <c r="F640" s="2">
         <v>46125</v>
@@ -33326,7 +33326,7 @@
         <v>1303</v>
       </c>
       <c r="C642" t="s">
-        <v>1541</v>
+        <v>1542</v>
       </c>
       <c r="F642" s="2">
         <v>45938</v>
@@ -33428,7 +33428,7 @@
         <v>1306</v>
       </c>
       <c r="C645" t="s">
-        <v>1514</v>
+        <v>1515</v>
       </c>
       <c r="F645" s="2">
         <v>45740</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-06-17 14:30:04
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -4273,7 +4273,7 @@
     <t>27/02/2025</t>
   </si>
   <si>
-    <t>08/05/2026</t>
+    <t>15/06/2026</t>
   </si>
   <si>
     <t>21/05/2025</t>
@@ -13533,7 +13533,7 @@
         <v>1419</v>
       </c>
       <c r="F26" s="2">
-        <v>46169</v>
+        <v>46190</v>
       </c>
       <c r="G26" t="s">
         <v>1776</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-08 10:30:04
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -33831,10 +33831,10 @@
         <v>1350</v>
       </c>
       <c r="C619" t="s">
-        <v>1613</v>
+        <v>1732</v>
       </c>
       <c r="F619" s="2">
-        <v>46149</v>
+        <v>46211</v>
       </c>
       <c r="G619" t="s">
         <v>1845</v>

</xml_diff>

<commit_message>
Add backlog, prod, and saida_sem_it - 2026-07-31 18:30:03
</commit_message>
<xml_diff>
--- a/SaidaSemITGATEAutoCompleto.xlsx
+++ b/SaidaSemITGATEAutoCompleto.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7124" uniqueCount="3637">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7126" uniqueCount="3637">
   <si>
     <t>PROCEDIMENTO_SEI</t>
   </si>
@@ -1600,9 +1600,6 @@
     <t>20.22.0001.0007823.2025-55</t>
   </si>
   <si>
-    <t>20.22.0001.0043118.2025-18</t>
-  </si>
-  <si>
     <t>20.22.0001.0056255.2025-48</t>
   </si>
   <si>
@@ -1936,6 +1933,9 @@
     <t>20.22.0001.0067524.2025-74</t>
   </si>
   <si>
+    <t>20.22.0001.0049964.2026-55</t>
+  </si>
+  <si>
     <t>20.22.0001.0076373.2025-62</t>
   </si>
   <si>
@@ -3847,9 +3847,6 @@
     <t>2025.0108</t>
   </si>
   <si>
-    <t>2025.0755</t>
-  </si>
-  <si>
     <t>2025.1006</t>
   </si>
   <si>
@@ -4183,6 +4180,9 @@
     <t>2025.1230</t>
   </si>
   <si>
+    <t>2026.0838</t>
+  </si>
+  <si>
     <t>2025.1382</t>
   </si>
   <si>
@@ -6376,31 +6376,31 @@
     <t>PROMOTORIA DE JUSTIÇA DE FAMÍLIA DE RESENDE</t>
   </si>
   <si>
+    <t>1ª PROMOTORIA DE JUSTIÇA DE SEROPÉDICA</t>
+  </si>
+  <si>
+    <t>1ª PROMOTORIA DE JUSTIÇA CÍVEL DE NOVA IGUAÇU - MESQUITA</t>
+  </si>
+  <si>
+    <t>7ª PROMOTORIA DE JUSTIÇA DE FAZENDA PÚBLICA DA CAPITAL</t>
+  </si>
+  <si>
+    <t>2ª PROMOTORIA DE JUSTIÇA DE TUTELA COLETIVA DE DEFESA DO MEIO AMBIENTE E DO PATRIMÔNIO CULTURAL DA CAPITAL</t>
+  </si>
+  <si>
+    <t>1ª PROMOTORIA DE JUSTIÇA DE TUTELA COLETIVA DO NÚCLEO CAMPOS DOS GOYTACAZES</t>
+  </si>
+  <si>
+    <t>PROMOTORIA DE JUSTIÇA DE FAMÍLIA, DA INFÂNCIA E DA JUVENTUDE DE TRÊS RIOS</t>
+  </si>
+  <si>
+    <t>4ª PROMOTORIA DE JUSTIÇA DA PESSOA IDOSA DA CAPITAL</t>
+  </si>
+  <si>
+    <t>PROMOTORIA DE JUSTIÇA DA INFÂNCIA E DA JUVENTUDE DE TERESÓPOLIS</t>
+  </si>
+  <si>
     <t>PROMOTORIA DE JUSTIÇA DE TUTELA COLETIVA DA PESSOA COM DEFICIÊNCIA DA CAPITAL</t>
-  </si>
-  <si>
-    <t>1ª PROMOTORIA DE JUSTIÇA DE SEROPÉDICA</t>
-  </si>
-  <si>
-    <t>1ª PROMOTORIA DE JUSTIÇA CÍVEL DE NOVA IGUAÇU - MESQUITA</t>
-  </si>
-  <si>
-    <t>7ª PROMOTORIA DE JUSTIÇA DE FAZENDA PÚBLICA DA CAPITAL</t>
-  </si>
-  <si>
-    <t>2ª PROMOTORIA DE JUSTIÇA DE TUTELA COLETIVA DE DEFESA DO MEIO AMBIENTE E DO PATRIMÔNIO CULTURAL DA CAPITAL</t>
-  </si>
-  <si>
-    <t>1ª PROMOTORIA DE JUSTIÇA DE TUTELA COLETIVA DO NÚCLEO CAMPOS DOS GOYTACAZES</t>
-  </si>
-  <si>
-    <t>PROMOTORIA DE JUSTIÇA DE FAMÍLIA, DA INFÂNCIA E DA JUVENTUDE DE TRÊS RIOS</t>
-  </si>
-  <si>
-    <t>4ª PROMOTORIA DE JUSTIÇA DA PESSOA IDOSA DA CAPITAL</t>
-  </si>
-  <si>
-    <t>PROMOTORIA DE JUSTIÇA DA INFÂNCIA E DA JUVENTUDE DE TERESÓPOLIS</t>
   </si>
   <si>
     <t>8ª PROMOTORIA DE JUSTIÇA DE TUTELA COLETIVA DE DEFESA DA CIDADANIA DA CAPITAL</t>
@@ -9560,9 +9560,6 @@
     <t>Solicito os bons préstimos no sentido de informar se é possível confeccionar IT contábil, diante dos novos esclarecimentos trazidos pela SEAS, ou se ratifica sua manifestação anterior.</t>
   </si>
   <si>
-    <t>Solicito apoio técnico do órgão na análise das informações prestadas pela SMAS, nos documentos de índexes 03910226 e 04402949, à luz da determinação exarada pelo Tribunal de Contas do Município no Processo TCM nº 040.100934.2019, especificamente no que diz respeito ao serviços destinados às pessoas com deficiência, de modo que seja indicado se as determinações do TCM foram cumpridas pelo MRJ, apontando-se, caso negativo, quais as pendências e as possíveis formas de regularização. Solicita-se, ainda, seja esclarecido se é possível concluir pela observância da Lei 13.019/2014 nos instrumentos firmados pelo MRJ com as entidades que compõe a RHC. Frisa-se que a SAT segue acompanhada da documentação constante de fls. 18/200 do volume I e de fls. 201/288 do volume II, além do despacho do índex 02202433.</t>
-  </si>
-  <si>
     <t>Análise da economicidade e regularidade da contratação do serviço de hospedagem para pessoas em situação de rua durante a pandemia de COVID-19, considerando o
 contexto emergencial, para que responda os quesitos iniciais abaixo indicados:
 1 - Análise de Preço e Mercado
@@ -10292,6 +10289,9 @@
     <t>Encaminhe as últimas respostas da Secretaria Municipal de Assistência Social de Magé ao GATE para complementação à IT nº 398/2025 a fim de verificar se as irregularidades antes constatadas foram sanadas pelos Municípios.</t>
   </si>
   <si>
+    <t>Análise das manifestações dos réus de ids 286073242 e 289938002, em resposta à IT 329/2026 do GATE, especialmente quanto à proposta de formalização de negócio jurídico para realização de perícia (privada) acerca de suposto desvio de rio.</t>
+  </si>
+  <si>
     <t>A solicitação de análise técnica ao GATE justifica-se pela necessidade de apurar e quantificar o dano ao erário decorrente do uso indevido do terminal rodoviário de Itaguaí, conforme indícios constantes dos autos. A apuração demanda avaliação técnica especializada, a fim de identificar o valor econômico do prejuízo ao erário municipal.</t>
   </si>
   <si>
@@ -12546,9 +12546,6 @@
     <t>https://sei.mprj.mp.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=4427641&amp;id_documento=4427642</t>
   </si>
   <si>
-    <t>https://sei.mprj.mp.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=4886904&amp;id_documento=4886905</t>
-  </si>
-  <si>
     <t>https://sei.mprj.mp.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=5069914&amp;id_documento=5069915</t>
   </si>
   <si>
@@ -12880,6 +12877,9 @@
   </si>
   <si>
     <t>https://sei.mprj.mp.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=5227432&amp;id_documento=5227433</t>
+  </si>
+  <si>
+    <t>https://sei.mprj.mp.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=6309470&amp;id_documento=6309471</t>
   </si>
   <si>
     <t>https://sei.mprj.mp.br/sei/controlador.php?acao=procedimento_trabalhar&amp;id_procedimento=5352423&amp;id_documento=5352424</t>
@@ -30904,19 +30904,19 @@
         <v>1277</v>
       </c>
       <c r="C518" t="s">
-        <v>1732</v>
+        <v>1802</v>
       </c>
       <c r="F518" s="2">
-        <v>45923</v>
+        <v>45994</v>
       </c>
       <c r="G518" t="s">
-        <v>1916</v>
+        <v>1918</v>
       </c>
       <c r="H518" t="s">
-        <v>1925</v>
+        <v>1924</v>
       </c>
       <c r="I518" t="s">
-        <v>2120</v>
+        <v>2039</v>
       </c>
       <c r="J518" t="s">
         <v>2142</v>
@@ -30936,19 +30936,19 @@
         <v>1278</v>
       </c>
       <c r="C519" t="s">
-        <v>1802</v>
+        <v>1715</v>
       </c>
       <c r="F519" s="2">
-        <v>45994</v>
+        <v>46090</v>
       </c>
       <c r="G519" t="s">
-        <v>1918</v>
+        <v>1916</v>
       </c>
       <c r="H519" t="s">
         <v>1924</v>
       </c>
       <c r="I519" t="s">
-        <v>2039</v>
+        <v>2050</v>
       </c>
       <c r="J519" t="s">
         <v>2142</v>
@@ -30968,19 +30968,19 @@
         <v>1279</v>
       </c>
       <c r="C520" t="s">
-        <v>1715</v>
+        <v>1803</v>
       </c>
       <c r="F520" s="2">
-        <v>46090</v>
+        <v>46188</v>
       </c>
       <c r="G520" t="s">
         <v>1916</v>
       </c>
       <c r="H520" t="s">
-        <v>1924</v>
+        <v>1923</v>
       </c>
       <c r="I520" t="s">
-        <v>2050</v>
+        <v>2020</v>
       </c>
       <c r="J520" t="s">
         <v>2142</v>
@@ -31000,19 +31000,19 @@
         <v>1280</v>
       </c>
       <c r="C521" t="s">
-        <v>1803</v>
+        <v>1569</v>
       </c>
       <c r="F521" s="2">
-        <v>46188</v>
+        <v>45996</v>
       </c>
       <c r="G521" t="s">
         <v>1916</v>
       </c>
       <c r="H521" t="s">
-        <v>1923</v>
+        <v>1926</v>
       </c>
       <c r="I521" t="s">
-        <v>2020</v>
+        <v>2120</v>
       </c>
       <c r="J521" t="s">
         <v>2142</v>
@@ -31032,19 +31032,19 @@
         <v>1281</v>
       </c>
       <c r="C522" t="s">
-        <v>1569</v>
+        <v>1804</v>
       </c>
       <c r="F522" s="2">
-        <v>45996</v>
+        <v>45673</v>
       </c>
       <c r="G522" t="s">
         <v>1916</v>
       </c>
       <c r="H522" t="s">
-        <v>1926</v>
+        <v>1923</v>
       </c>
       <c r="I522" t="s">
-        <v>2121</v>
+        <v>2012</v>
       </c>
       <c r="J522" t="s">
         <v>2142</v>
@@ -31064,19 +31064,19 @@
         <v>1282</v>
       </c>
       <c r="C523" t="s">
-        <v>1804</v>
+        <v>1805</v>
       </c>
       <c r="F523" s="2">
-        <v>45673</v>
+        <v>45919</v>
       </c>
       <c r="G523" t="s">
         <v>1916</v>
       </c>
       <c r="H523" t="s">
-        <v>1923</v>
+        <v>1924</v>
       </c>
       <c r="I523" t="s">
-        <v>2012</v>
+        <v>1996</v>
       </c>
       <c r="J523" t="s">
         <v>2142</v>
@@ -31096,19 +31096,19 @@
         <v>1283</v>
       </c>
       <c r="C524" t="s">
-        <v>1805</v>
+        <v>1694</v>
       </c>
       <c r="F524" s="2">
-        <v>45919</v>
+        <v>45946</v>
       </c>
       <c r="G524" t="s">
         <v>1916</v>
       </c>
       <c r="H524" t="s">
-        <v>1924</v>
+        <v>1923</v>
       </c>
       <c r="I524" t="s">
-        <v>1996</v>
+        <v>1988</v>
       </c>
       <c r="J524" t="s">
         <v>2142</v>
@@ -31128,10 +31128,10 @@
         <v>1284</v>
       </c>
       <c r="C525" t="s">
-        <v>1694</v>
+        <v>1604</v>
       </c>
       <c r="F525" s="2">
-        <v>45946</v>
+        <v>45838</v>
       </c>
       <c r="G525" t="s">
         <v>1916</v>
@@ -31140,7 +31140,7 @@
         <v>1923</v>
       </c>
       <c r="I525" t="s">
-        <v>1988</v>
+        <v>2099</v>
       </c>
       <c r="J525" t="s">
         <v>2142</v>
@@ -31160,19 +31160,25 @@
         <v>1285</v>
       </c>
       <c r="C526" t="s">
-        <v>1604</v>
+        <v>1806</v>
+      </c>
+      <c r="D526" t="s">
+        <v>1688</v>
+      </c>
+      <c r="E526" t="s">
+        <v>1688</v>
       </c>
       <c r="F526" s="2">
-        <v>45838</v>
+        <v>45994</v>
       </c>
       <c r="G526" t="s">
         <v>1916</v>
       </c>
       <c r="H526" t="s">
-        <v>1923</v>
+        <v>1942</v>
       </c>
       <c r="I526" t="s">
-        <v>2099</v>
+        <v>1976</v>
       </c>
       <c r="J526" t="s">
         <v>2142</v>
@@ -31192,25 +31198,25 @@
         <v>1286</v>
       </c>
       <c r="C527" t="s">
-        <v>1806</v>
+        <v>1528</v>
       </c>
       <c r="D527" t="s">
-        <v>1688</v>
+        <v>1513</v>
       </c>
       <c r="E527" t="s">
-        <v>1688</v>
+        <v>1913</v>
       </c>
       <c r="F527" s="2">
-        <v>45994</v>
+        <v>45772</v>
       </c>
       <c r="G527" t="s">
         <v>1916</v>
       </c>
       <c r="H527" t="s">
-        <v>1942</v>
+        <v>1952</v>
       </c>
       <c r="I527" t="s">
-        <v>1976</v>
+        <v>1978</v>
       </c>
       <c r="J527" t="s">
         <v>2142</v>
@@ -31230,25 +31236,19 @@
         <v>1287</v>
       </c>
       <c r="C528" t="s">
-        <v>1528</v>
-      </c>
-      <c r="D528" t="s">
-        <v>1513</v>
-      </c>
-      <c r="E528" t="s">
-        <v>1913</v>
+        <v>1807</v>
       </c>
       <c r="F528" s="2">
-        <v>45772</v>
+        <v>45989</v>
       </c>
       <c r="G528" t="s">
-        <v>1916</v>
+        <v>1917</v>
       </c>
       <c r="H528" t="s">
-        <v>1952</v>
+        <v>1926</v>
       </c>
       <c r="I528" t="s">
-        <v>1978</v>
+        <v>2121</v>
       </c>
       <c r="J528" t="s">
         <v>2142</v>
@@ -31268,19 +31268,22 @@
         <v>1288</v>
       </c>
       <c r="C529" t="s">
-        <v>1807</v>
+        <v>1520</v>
+      </c>
+      <c r="D529" t="s">
+        <v>1883</v>
       </c>
       <c r="F529" s="2">
-        <v>45989</v>
+        <v>46147</v>
       </c>
       <c r="G529" t="s">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="H529" t="s">
-        <v>1926</v>
+        <v>1932</v>
       </c>
       <c r="I529" t="s">
-        <v>2122</v>
+        <v>1982</v>
       </c>
       <c r="J529" t="s">
         <v>2142</v>
@@ -31300,22 +31303,19 @@
         <v>1289</v>
       </c>
       <c r="C530" t="s">
-        <v>1520</v>
-      </c>
-      <c r="D530" t="s">
-        <v>1883</v>
+        <v>1607</v>
       </c>
       <c r="F530" s="2">
-        <v>46147</v>
+        <v>46184</v>
       </c>
       <c r="G530" t="s">
         <v>1916</v>
       </c>
       <c r="H530" t="s">
-        <v>1932</v>
+        <v>1924</v>
       </c>
       <c r="I530" t="s">
-        <v>1982</v>
+        <v>2018</v>
       </c>
       <c r="J530" t="s">
         <v>2142</v>
@@ -31335,19 +31335,19 @@
         <v>1290</v>
       </c>
       <c r="C531" t="s">
-        <v>1607</v>
+        <v>1690</v>
       </c>
       <c r="F531" s="2">
-        <v>46184</v>
+        <v>46049</v>
       </c>
       <c r="G531" t="s">
         <v>1916</v>
       </c>
       <c r="H531" t="s">
-        <v>1924</v>
+        <v>1923</v>
       </c>
       <c r="I531" t="s">
-        <v>2018</v>
+        <v>1980</v>
       </c>
       <c r="J531" t="s">
         <v>2142</v>
@@ -31367,19 +31367,25 @@
         <v>1291</v>
       </c>
       <c r="C532" t="s">
-        <v>1690</v>
+        <v>1808</v>
+      </c>
+      <c r="D532" t="s">
+        <v>1889</v>
+      </c>
+      <c r="E532" t="s">
+        <v>1889</v>
       </c>
       <c r="F532" s="2">
-        <v>46049</v>
+        <v>46227</v>
       </c>
       <c r="G532" t="s">
-        <v>1916</v>
+        <v>1917</v>
       </c>
       <c r="H532" t="s">
-        <v>1923</v>
+        <v>1941</v>
       </c>
       <c r="I532" t="s">
-        <v>1980</v>
+        <v>2001</v>
       </c>
       <c r="J532" t="s">
         <v>2142</v>
@@ -31399,25 +31405,25 @@
         <v>1292</v>
       </c>
       <c r="C533" t="s">
-        <v>1808</v>
+        <v>1634</v>
       </c>
       <c r="D533" t="s">
-        <v>1889</v>
+        <v>1568</v>
       </c>
       <c r="E533" t="s">
-        <v>1889</v>
+        <v>1826</v>
       </c>
       <c r="F533" s="2">
-        <v>46227</v>
+        <v>45924</v>
       </c>
       <c r="G533" t="s">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="H533" t="s">
-        <v>1941</v>
+        <v>1923</v>
       </c>
       <c r="I533" t="s">
-        <v>2001</v>
+        <v>2011</v>
       </c>
       <c r="J533" t="s">
         <v>2142</v>
@@ -31437,16 +31443,10 @@
         <v>1293</v>
       </c>
       <c r="C534" t="s">
-        <v>1634</v>
-      </c>
-      <c r="D534" t="s">
-        <v>1568</v>
-      </c>
-      <c r="E534" t="s">
-        <v>1826</v>
+        <v>1638</v>
       </c>
       <c r="F534" s="2">
-        <v>45924</v>
+        <v>45891</v>
       </c>
       <c r="G534" t="s">
         <v>1916</v>
@@ -31455,7 +31455,7 @@
         <v>1923</v>
       </c>
       <c r="I534" t="s">
-        <v>2011</v>
+        <v>2005</v>
       </c>
       <c r="J534" t="s">
         <v>2142</v>
@@ -31475,19 +31475,19 @@
         <v>1294</v>
       </c>
       <c r="C535" t="s">
-        <v>1638</v>
+        <v>1694</v>
       </c>
       <c r="F535" s="2">
-        <v>45891</v>
+        <v>45812</v>
       </c>
       <c r="G535" t="s">
         <v>1916</v>
       </c>
       <c r="H535" t="s">
-        <v>1923</v>
+        <v>1924</v>
       </c>
       <c r="I535" t="s">
-        <v>2005</v>
+        <v>2011</v>
       </c>
       <c r="J535" t="s">
         <v>2142</v>
@@ -31507,22 +31507,28 @@
         <v>1295</v>
       </c>
       <c r="C536" t="s">
-        <v>1694</v>
+        <v>1561</v>
+      </c>
+      <c r="D536" t="s">
+        <v>1659</v>
+      </c>
+      <c r="E536" t="s">
+        <v>1659</v>
       </c>
       <c r="F536" s="2">
-        <v>45812</v>
+        <v>46048</v>
       </c>
       <c r="G536" t="s">
-        <v>1916</v>
+        <v>1917</v>
       </c>
       <c r="H536" t="s">
-        <v>1924</v>
+        <v>1969</v>
       </c>
       <c r="I536" t="s">
-        <v>2011</v>
+        <v>2122</v>
       </c>
       <c r="J536" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K536" t="s">
         <v>2675</v>
@@ -31539,25 +31545,25 @@
         <v>1296</v>
       </c>
       <c r="C537" t="s">
-        <v>1561</v>
+        <v>1603</v>
       </c>
       <c r="D537" t="s">
-        <v>1659</v>
+        <v>1741</v>
       </c>
       <c r="E537" t="s">
-        <v>1659</v>
+        <v>1547</v>
       </c>
       <c r="F537" s="2">
-        <v>46048</v>
+        <v>45908</v>
       </c>
       <c r="G537" t="s">
         <v>1917</v>
       </c>
       <c r="H537" t="s">
-        <v>1969</v>
+        <v>1970</v>
       </c>
       <c r="I537" t="s">
-        <v>2123</v>
+        <v>2051</v>
       </c>
       <c r="J537" t="s">
         <v>2143</v>
@@ -31577,28 +31583,22 @@
         <v>1297</v>
       </c>
       <c r="C538" t="s">
-        <v>1603</v>
-      </c>
-      <c r="D538" t="s">
-        <v>1741</v>
-      </c>
-      <c r="E538" t="s">
-        <v>1547</v>
+        <v>1739</v>
       </c>
       <c r="F538" s="2">
-        <v>45908</v>
+        <v>46113</v>
       </c>
       <c r="G538" t="s">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="H538" t="s">
-        <v>1970</v>
+        <v>1923</v>
       </c>
       <c r="I538" t="s">
-        <v>2051</v>
+        <v>2009</v>
       </c>
       <c r="J538" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K538" t="s">
         <v>2677</v>
@@ -31615,19 +31615,19 @@
         <v>1298</v>
       </c>
       <c r="C539" t="s">
-        <v>1739</v>
+        <v>1760</v>
       </c>
       <c r="F539" s="2">
-        <v>46113</v>
+        <v>45693</v>
       </c>
       <c r="G539" t="s">
         <v>1916</v>
       </c>
       <c r="H539" t="s">
-        <v>1923</v>
+        <v>1924</v>
       </c>
       <c r="I539" t="s">
-        <v>2009</v>
+        <v>1978</v>
       </c>
       <c r="J539" t="s">
         <v>2142</v>
@@ -31647,22 +31647,22 @@
         <v>1299</v>
       </c>
       <c r="C540" t="s">
-        <v>1760</v>
+        <v>1809</v>
       </c>
       <c r="F540" s="2">
-        <v>45693</v>
+        <v>45735</v>
       </c>
       <c r="G540" t="s">
         <v>1916</v>
       </c>
       <c r="H540" t="s">
-        <v>1924</v>
+        <v>1938</v>
       </c>
       <c r="I540" t="s">
-        <v>1978</v>
+        <v>2123</v>
       </c>
       <c r="J540" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K540" t="s">
         <v>2679</v>
@@ -31679,22 +31679,22 @@
         <v>1300</v>
       </c>
       <c r="C541" t="s">
-        <v>1809</v>
+        <v>1798</v>
       </c>
       <c r="F541" s="2">
-        <v>45735</v>
+        <v>46189</v>
       </c>
       <c r="G541" t="s">
         <v>1916</v>
       </c>
       <c r="H541" t="s">
-        <v>1938</v>
+        <v>1923</v>
       </c>
       <c r="I541" t="s">
-        <v>2124</v>
+        <v>2007</v>
       </c>
       <c r="J541" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K541" t="s">
         <v>2680</v>
@@ -31711,19 +31711,25 @@
         <v>1301</v>
       </c>
       <c r="C542" t="s">
-        <v>1798</v>
+        <v>1537</v>
+      </c>
+      <c r="D542" t="s">
+        <v>1830</v>
+      </c>
+      <c r="E542" t="s">
+        <v>1830</v>
       </c>
       <c r="F542" s="2">
-        <v>46189</v>
+        <v>46118</v>
       </c>
       <c r="G542" t="s">
         <v>1916</v>
       </c>
       <c r="H542" t="s">
-        <v>1923</v>
+        <v>1943</v>
       </c>
       <c r="I542" t="s">
-        <v>2007</v>
+        <v>2030</v>
       </c>
       <c r="J542" t="s">
         <v>2142</v>
@@ -31743,25 +31749,19 @@
         <v>1302</v>
       </c>
       <c r="C543" t="s">
-        <v>1537</v>
-      </c>
-      <c r="D543" t="s">
-        <v>1830</v>
-      </c>
-      <c r="E543" t="s">
-        <v>1830</v>
+        <v>1767</v>
       </c>
       <c r="F543" s="2">
-        <v>46118</v>
+        <v>45812</v>
       </c>
       <c r="G543" t="s">
         <v>1916</v>
       </c>
       <c r="H543" t="s">
-        <v>1943</v>
+        <v>1924</v>
       </c>
       <c r="I543" t="s">
-        <v>2030</v>
+        <v>2124</v>
       </c>
       <c r="J543" t="s">
         <v>2142</v>
@@ -31781,22 +31781,22 @@
         <v>1303</v>
       </c>
       <c r="C544" t="s">
-        <v>1767</v>
+        <v>1532</v>
       </c>
       <c r="F544" s="2">
-        <v>45812</v>
+        <v>46204</v>
       </c>
       <c r="G544" t="s">
         <v>1916</v>
       </c>
       <c r="H544" t="s">
-        <v>1924</v>
+        <v>1923</v>
       </c>
       <c r="I544" t="s">
-        <v>2125</v>
+        <v>2011</v>
       </c>
       <c r="J544" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K544" t="s">
         <v>2683</v>
@@ -31813,22 +31813,25 @@
         <v>1304</v>
       </c>
       <c r="C545" t="s">
-        <v>1532</v>
+        <v>1663</v>
+      </c>
+      <c r="D545" t="s">
+        <v>1678</v>
       </c>
       <c r="F545" s="2">
-        <v>46204</v>
+        <v>45709</v>
       </c>
       <c r="G545" t="s">
-        <v>1916</v>
+        <v>1919</v>
       </c>
       <c r="H545" t="s">
-        <v>1923</v>
+        <v>1925</v>
       </c>
       <c r="I545" t="s">
-        <v>2011</v>
+        <v>2073</v>
       </c>
       <c r="J545" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K545" t="s">
         <v>2684</v>
@@ -31845,22 +31848,19 @@
         <v>1305</v>
       </c>
       <c r="C546" t="s">
-        <v>1663</v>
-      </c>
-      <c r="D546" t="s">
-        <v>1678</v>
+        <v>1606</v>
       </c>
       <c r="F546" s="2">
-        <v>45709</v>
+        <v>46148</v>
       </c>
       <c r="G546" t="s">
-        <v>1919</v>
+        <v>1916</v>
       </c>
       <c r="H546" t="s">
-        <v>1925</v>
+        <v>1923</v>
       </c>
       <c r="I546" t="s">
-        <v>2073</v>
+        <v>2012</v>
       </c>
       <c r="J546" t="s">
         <v>2142</v>
@@ -31880,19 +31880,22 @@
         <v>1306</v>
       </c>
       <c r="C547" t="s">
-        <v>1606</v>
+        <v>1810</v>
+      </c>
+      <c r="D547" t="s">
+        <v>1515</v>
       </c>
       <c r="F547" s="2">
-        <v>46148</v>
+        <v>46211</v>
       </c>
       <c r="G547" t="s">
         <v>1916</v>
       </c>
       <c r="H547" t="s">
-        <v>1923</v>
+        <v>1932</v>
       </c>
       <c r="I547" t="s">
-        <v>2012</v>
+        <v>2125</v>
       </c>
       <c r="J547" t="s">
         <v>2142</v>
@@ -31912,22 +31915,19 @@
         <v>1307</v>
       </c>
       <c r="C548" t="s">
-        <v>1810</v>
-      </c>
-      <c r="D548" t="s">
-        <v>1515</v>
+        <v>1752</v>
       </c>
       <c r="F548" s="2">
-        <v>46211</v>
+        <v>46044</v>
       </c>
       <c r="G548" t="s">
         <v>1916</v>
       </c>
       <c r="H548" t="s">
-        <v>1932</v>
+        <v>1923</v>
       </c>
       <c r="I548" t="s">
-        <v>2126</v>
+        <v>2029</v>
       </c>
       <c r="J548" t="s">
         <v>2142</v>
@@ -31947,19 +31947,19 @@
         <v>1308</v>
       </c>
       <c r="C549" t="s">
-        <v>1752</v>
+        <v>1521</v>
       </c>
       <c r="F549" s="2">
-        <v>46044</v>
+        <v>45994</v>
       </c>
       <c r="G549" t="s">
         <v>1916</v>
       </c>
       <c r="H549" t="s">
-        <v>1923</v>
+        <v>1921</v>
       </c>
       <c r="I549" t="s">
-        <v>2029</v>
+        <v>2013</v>
       </c>
       <c r="J549" t="s">
         <v>2142</v>
@@ -31979,22 +31979,28 @@
         <v>1309</v>
       </c>
       <c r="C550" t="s">
-        <v>1521</v>
+        <v>1811</v>
+      </c>
+      <c r="D550" t="s">
+        <v>1703</v>
+      </c>
+      <c r="E550" t="s">
+        <v>1707</v>
       </c>
       <c r="F550" s="2">
-        <v>45994</v>
+        <v>46034</v>
       </c>
       <c r="G550" t="s">
         <v>1916</v>
       </c>
       <c r="H550" t="s">
-        <v>1921</v>
+        <v>1929</v>
       </c>
       <c r="I550" t="s">
-        <v>2013</v>
+        <v>1992</v>
       </c>
       <c r="J550" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K550" t="s">
         <v>2689</v>
@@ -32011,25 +32017,25 @@
         <v>1310</v>
       </c>
       <c r="C551" t="s">
-        <v>1811</v>
+        <v>1644</v>
       </c>
       <c r="D551" t="s">
-        <v>1703</v>
+        <v>1767</v>
       </c>
       <c r="E551" t="s">
-        <v>1707</v>
+        <v>1767</v>
       </c>
       <c r="F551" s="2">
-        <v>46034</v>
+        <v>45811</v>
       </c>
       <c r="G551" t="s">
         <v>1916</v>
       </c>
       <c r="H551" t="s">
-        <v>1929</v>
+        <v>1943</v>
       </c>
       <c r="I551" t="s">
-        <v>1992</v>
+        <v>2097</v>
       </c>
       <c r="J551" t="s">
         <v>2143</v>
@@ -32049,25 +32055,19 @@
         <v>1311</v>
       </c>
       <c r="C552" t="s">
-        <v>1644</v>
-      </c>
-      <c r="D552" t="s">
-        <v>1767</v>
-      </c>
-      <c r="E552" t="s">
-        <v>1767</v>
+        <v>1543</v>
       </c>
       <c r="F552" s="2">
-        <v>45811</v>
+        <v>46167</v>
       </c>
       <c r="G552" t="s">
         <v>1916</v>
       </c>
       <c r="H552" t="s">
-        <v>1943</v>
+        <v>1923</v>
       </c>
       <c r="I552" t="s">
-        <v>2097</v>
+        <v>1988</v>
       </c>
       <c r="J552" t="s">
         <v>2143</v>
@@ -32087,22 +32087,22 @@
         <v>1312</v>
       </c>
       <c r="C553" t="s">
-        <v>1543</v>
+        <v>1678</v>
       </c>
       <c r="F553" s="2">
-        <v>46167</v>
+        <v>45680</v>
       </c>
       <c r="G553" t="s">
         <v>1916</v>
       </c>
       <c r="H553" t="s">
-        <v>1923</v>
+        <v>1924</v>
       </c>
       <c r="I553" t="s">
-        <v>1988</v>
+        <v>2021</v>
       </c>
       <c r="J553" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K553" t="s">
         <v>2692</v>
@@ -32119,10 +32119,10 @@
         <v>1313</v>
       </c>
       <c r="C554" t="s">
-        <v>1678</v>
+        <v>1746</v>
       </c>
       <c r="F554" s="2">
-        <v>45680</v>
+        <v>45754</v>
       </c>
       <c r="G554" t="s">
         <v>1916</v>
@@ -32131,7 +32131,7 @@
         <v>1924</v>
       </c>
       <c r="I554" t="s">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="J554" t="s">
         <v>2142</v>
@@ -32151,19 +32151,19 @@
         <v>1314</v>
       </c>
       <c r="C555" t="s">
-        <v>1746</v>
+        <v>1563</v>
       </c>
       <c r="F555" s="2">
-        <v>45754</v>
+        <v>46160</v>
       </c>
       <c r="G555" t="s">
         <v>1916</v>
       </c>
       <c r="H555" t="s">
-        <v>1924</v>
+        <v>1923</v>
       </c>
       <c r="I555" t="s">
-        <v>2022</v>
+        <v>2018</v>
       </c>
       <c r="J555" t="s">
         <v>2142</v>
@@ -32183,22 +32183,22 @@
         <v>1315</v>
       </c>
       <c r="C556" t="s">
-        <v>1563</v>
+        <v>1737</v>
       </c>
       <c r="F556" s="2">
-        <v>46160</v>
+        <v>45854</v>
       </c>
       <c r="G556" t="s">
         <v>1916</v>
       </c>
       <c r="H556" t="s">
-        <v>1923</v>
+        <v>1924</v>
       </c>
       <c r="I556" t="s">
-        <v>2018</v>
+        <v>1980</v>
       </c>
       <c r="J556" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K556" t="s">
         <v>2695</v>
@@ -32215,22 +32215,25 @@
         <v>1316</v>
       </c>
       <c r="C557" t="s">
-        <v>1737</v>
+        <v>1768</v>
+      </c>
+      <c r="D557" t="s">
+        <v>1890</v>
       </c>
       <c r="F557" s="2">
-        <v>45854</v>
+        <v>45782</v>
       </c>
       <c r="G557" t="s">
         <v>1916</v>
       </c>
       <c r="H557" t="s">
-        <v>1924</v>
+        <v>1926</v>
       </c>
       <c r="I557" t="s">
-        <v>1980</v>
+        <v>2031</v>
       </c>
       <c r="J557" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K557" t="s">
         <v>2696</v>
@@ -32247,13 +32250,10 @@
         <v>1317</v>
       </c>
       <c r="C558" t="s">
-        <v>1768</v>
-      </c>
-      <c r="D558" t="s">
-        <v>1890</v>
+        <v>1516</v>
       </c>
       <c r="F558" s="2">
-        <v>45782</v>
+        <v>46010</v>
       </c>
       <c r="G558" t="s">
         <v>1916</v>
@@ -32262,7 +32262,7 @@
         <v>1926</v>
       </c>
       <c r="I558" t="s">
-        <v>2031</v>
+        <v>2041</v>
       </c>
       <c r="J558" t="s">
         <v>2142</v>
@@ -32282,10 +32282,10 @@
         <v>1318</v>
       </c>
       <c r="C559" t="s">
-        <v>1516</v>
+        <v>1644</v>
       </c>
       <c r="F559" s="2">
-        <v>46010</v>
+        <v>45812</v>
       </c>
       <c r="G559" t="s">
         <v>1916</v>
@@ -32294,7 +32294,7 @@
         <v>1926</v>
       </c>
       <c r="I559" t="s">
-        <v>2041</v>
+        <v>2097</v>
       </c>
       <c r="J559" t="s">
         <v>2142</v>
@@ -32314,22 +32314,28 @@
         <v>1319</v>
       </c>
       <c r="C560" t="s">
-        <v>1644</v>
+        <v>1676</v>
+      </c>
+      <c r="D560" t="s">
+        <v>1605</v>
+      </c>
+      <c r="E560" t="s">
+        <v>1605</v>
       </c>
       <c r="F560" s="2">
-        <v>45812</v>
+        <v>45884</v>
       </c>
       <c r="G560" t="s">
         <v>1916</v>
       </c>
       <c r="H560" t="s">
-        <v>1926</v>
+        <v>1924</v>
       </c>
       <c r="I560" t="s">
-        <v>2097</v>
+        <v>2062</v>
       </c>
       <c r="J560" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K560" t="s">
         <v>2699</v>
@@ -32346,28 +32352,22 @@
         <v>1320</v>
       </c>
       <c r="C561" t="s">
-        <v>1676</v>
-      </c>
-      <c r="D561" t="s">
-        <v>1605</v>
-      </c>
-      <c r="E561" t="s">
-        <v>1605</v>
+        <v>1805</v>
       </c>
       <c r="F561" s="2">
-        <v>45884</v>
+        <v>45995</v>
       </c>
       <c r="G561" t="s">
         <v>1916</v>
       </c>
       <c r="H561" t="s">
-        <v>1924</v>
+        <v>1923</v>
       </c>
       <c r="I561" t="s">
-        <v>2062</v>
+        <v>2009</v>
       </c>
       <c r="J561" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K561" t="s">
         <v>2700</v>
@@ -32384,19 +32384,25 @@
         <v>1321</v>
       </c>
       <c r="C562" t="s">
-        <v>1805</v>
+        <v>1613</v>
+      </c>
+      <c r="D562" t="s">
+        <v>1677</v>
+      </c>
+      <c r="E562" t="s">
+        <v>1677</v>
       </c>
       <c r="F562" s="2">
-        <v>45995</v>
+        <v>46167</v>
       </c>
       <c r="G562" t="s">
         <v>1916</v>
       </c>
       <c r="H562" t="s">
-        <v>1923</v>
+        <v>1932</v>
       </c>
       <c r="I562" t="s">
-        <v>2009</v>
+        <v>2124</v>
       </c>
       <c r="J562" t="s">
         <v>2142</v>
@@ -32416,28 +32422,22 @@
         <v>1322</v>
       </c>
       <c r="C563" t="s">
-        <v>1613</v>
-      </c>
-      <c r="D563" t="s">
-        <v>1677</v>
-      </c>
-      <c r="E563" t="s">
-        <v>1677</v>
+        <v>1710</v>
       </c>
       <c r="F563" s="2">
-        <v>46167</v>
+        <v>45704</v>
       </c>
       <c r="G563" t="s">
         <v>1916</v>
       </c>
       <c r="H563" t="s">
-        <v>1932</v>
+        <v>1924</v>
       </c>
       <c r="I563" t="s">
-        <v>2125</v>
+        <v>1979</v>
       </c>
       <c r="J563" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K563" t="s">
         <v>2702</v>
@@ -32454,22 +32454,28 @@
         <v>1323</v>
       </c>
       <c r="C564" t="s">
-        <v>1710</v>
+        <v>1729</v>
+      </c>
+      <c r="D564" t="s">
+        <v>1891</v>
+      </c>
+      <c r="E564" t="s">
+        <v>1891</v>
       </c>
       <c r="F564" s="2">
-        <v>45704</v>
+        <v>46181</v>
       </c>
       <c r="G564" t="s">
         <v>1916</v>
       </c>
       <c r="H564" t="s">
-        <v>1924</v>
+        <v>1923</v>
       </c>
       <c r="I564" t="s">
-        <v>1979</v>
+        <v>2048</v>
       </c>
       <c r="J564" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K564" t="s">
         <v>2703</v>
@@ -32486,25 +32492,19 @@
         <v>1324</v>
       </c>
       <c r="C565" t="s">
-        <v>1729</v>
-      </c>
-      <c r="D565" t="s">
-        <v>1891</v>
-      </c>
-      <c r="E565" t="s">
-        <v>1891</v>
+        <v>1795</v>
       </c>
       <c r="F565" s="2">
-        <v>46181</v>
+        <v>46204</v>
       </c>
       <c r="G565" t="s">
         <v>1916</v>
       </c>
       <c r="H565" t="s">
-        <v>1923</v>
+        <v>1942</v>
       </c>
       <c r="I565" t="s">
-        <v>2048</v>
+        <v>2029</v>
       </c>
       <c r="J565" t="s">
         <v>2142</v>
@@ -32524,19 +32524,19 @@
         <v>1325</v>
       </c>
       <c r="C566" t="s">
-        <v>1795</v>
+        <v>1732</v>
       </c>
       <c r="F566" s="2">
-        <v>46204</v>
+        <v>45853</v>
       </c>
       <c r="G566" t="s">
         <v>1916</v>
       </c>
       <c r="H566" t="s">
-        <v>1942</v>
+        <v>1926</v>
       </c>
       <c r="I566" t="s">
-        <v>2029</v>
+        <v>2076</v>
       </c>
       <c r="J566" t="s">
         <v>2142</v>
@@ -32556,19 +32556,19 @@
         <v>1326</v>
       </c>
       <c r="C567" t="s">
-        <v>1732</v>
+        <v>1518</v>
       </c>
       <c r="F567" s="2">
-        <v>45853</v>
+        <v>45705</v>
       </c>
       <c r="G567" t="s">
-        <v>1916</v>
+        <v>1919</v>
       </c>
       <c r="H567" t="s">
         <v>1926</v>
       </c>
       <c r="I567" t="s">
-        <v>2076</v>
+        <v>2126</v>
       </c>
       <c r="J567" t="s">
         <v>2142</v>
@@ -32588,19 +32588,19 @@
         <v>1327</v>
       </c>
       <c r="C568" t="s">
-        <v>1518</v>
+        <v>1669</v>
       </c>
       <c r="F568" s="2">
-        <v>45705</v>
+        <v>45862</v>
       </c>
       <c r="G568" t="s">
-        <v>1919</v>
+        <v>1916</v>
       </c>
       <c r="H568" t="s">
-        <v>1926</v>
+        <v>1924</v>
       </c>
       <c r="I568" t="s">
-        <v>2127</v>
+        <v>2011</v>
       </c>
       <c r="J568" t="s">
         <v>2142</v>
@@ -32620,19 +32620,25 @@
         <v>1328</v>
       </c>
       <c r="C569" t="s">
-        <v>1669</v>
+        <v>1519</v>
+      </c>
+      <c r="D569" t="s">
+        <v>1866</v>
+      </c>
+      <c r="E569" t="s">
+        <v>1844</v>
       </c>
       <c r="F569" s="2">
-        <v>45862</v>
+        <v>45992</v>
       </c>
       <c r="G569" t="s">
         <v>1916</v>
       </c>
       <c r="H569" t="s">
-        <v>1924</v>
+        <v>1930</v>
       </c>
       <c r="I569" t="s">
-        <v>2011</v>
+        <v>1983</v>
       </c>
       <c r="J569" t="s">
         <v>2142</v>
@@ -32652,25 +32658,19 @@
         <v>1329</v>
       </c>
       <c r="C570" t="s">
-        <v>1519</v>
-      </c>
-      <c r="D570" t="s">
-        <v>1866</v>
-      </c>
-      <c r="E570" t="s">
-        <v>1844</v>
+        <v>1812</v>
       </c>
       <c r="F570" s="2">
-        <v>45992</v>
+        <v>46010</v>
       </c>
       <c r="G570" t="s">
         <v>1916</v>
       </c>
       <c r="H570" t="s">
-        <v>1930</v>
+        <v>1923</v>
       </c>
       <c r="I570" t="s">
-        <v>1983</v>
+        <v>2023</v>
       </c>
       <c r="J570" t="s">
         <v>2142</v>
@@ -32690,19 +32690,22 @@
         <v>1330</v>
       </c>
       <c r="C571" t="s">
-        <v>1812</v>
+        <v>1813</v>
+      </c>
+      <c r="D571" t="s">
+        <v>1601</v>
       </c>
       <c r="F571" s="2">
-        <v>46010</v>
+        <v>45972</v>
       </c>
       <c r="G571" t="s">
         <v>1916</v>
       </c>
       <c r="H571" t="s">
-        <v>1923</v>
+        <v>1945</v>
       </c>
       <c r="I571" t="s">
-        <v>2023</v>
+        <v>2020</v>
       </c>
       <c r="J571" t="s">
         <v>2142</v>
@@ -32722,22 +32725,19 @@
         <v>1331</v>
       </c>
       <c r="C572" t="s">
-        <v>1813</v>
-      </c>
-      <c r="D572" t="s">
-        <v>1601</v>
+        <v>1806</v>
       </c>
       <c r="F572" s="2">
-        <v>45972</v>
+        <v>45849</v>
       </c>
       <c r="G572" t="s">
         <v>1916</v>
       </c>
       <c r="H572" t="s">
-        <v>1945</v>
+        <v>1924</v>
       </c>
       <c r="I572" t="s">
-        <v>2020</v>
+        <v>1976</v>
       </c>
       <c r="J572" t="s">
         <v>2142</v>
@@ -32757,10 +32757,10 @@
         <v>1332</v>
       </c>
       <c r="C573" t="s">
-        <v>1806</v>
+        <v>1570</v>
       </c>
       <c r="F573" s="2">
-        <v>45849</v>
+        <v>45965</v>
       </c>
       <c r="G573" t="s">
         <v>1916</v>
@@ -32769,10 +32769,10 @@
         <v>1924</v>
       </c>
       <c r="I573" t="s">
-        <v>1976</v>
+        <v>2099</v>
       </c>
       <c r="J573" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K573" t="s">
         <v>2712</v>
@@ -32789,10 +32789,10 @@
         <v>1333</v>
       </c>
       <c r="C574" t="s">
-        <v>1570</v>
+        <v>1795</v>
       </c>
       <c r="F574" s="2">
-        <v>45965</v>
+        <v>46224</v>
       </c>
       <c r="G574" t="s">
         <v>1916</v>
@@ -32801,10 +32801,10 @@
         <v>1924</v>
       </c>
       <c r="I574" t="s">
-        <v>2099</v>
+        <v>2009</v>
       </c>
       <c r="J574" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K574" t="s">
         <v>2713</v>
@@ -32821,19 +32821,19 @@
         <v>1334</v>
       </c>
       <c r="C575" t="s">
-        <v>1795</v>
+        <v>1526</v>
       </c>
       <c r="F575" s="2">
-        <v>46224</v>
+        <v>45811</v>
       </c>
       <c r="G575" t="s">
-        <v>1916</v>
+        <v>1917</v>
       </c>
       <c r="H575" t="s">
-        <v>1924</v>
+        <v>1940</v>
       </c>
       <c r="I575" t="s">
-        <v>2009</v>
+        <v>1980</v>
       </c>
       <c r="J575" t="s">
         <v>2142</v>
@@ -32853,19 +32853,19 @@
         <v>1335</v>
       </c>
       <c r="C576" t="s">
-        <v>1526</v>
+        <v>1780</v>
       </c>
       <c r="F576" s="2">
-        <v>45811</v>
+        <v>46232</v>
       </c>
       <c r="G576" t="s">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="H576" t="s">
-        <v>1940</v>
+        <v>1923</v>
       </c>
       <c r="I576" t="s">
-        <v>1980</v>
+        <v>2034</v>
       </c>
       <c r="J576" t="s">
         <v>2142</v>
@@ -32885,19 +32885,19 @@
         <v>1336</v>
       </c>
       <c r="C577" t="s">
-        <v>1780</v>
+        <v>1814</v>
       </c>
       <c r="F577" s="2">
-        <v>46232</v>
+        <v>45811</v>
       </c>
       <c r="G577" t="s">
-        <v>1916</v>
+        <v>1918</v>
       </c>
       <c r="H577" t="s">
-        <v>1923</v>
+        <v>1924</v>
       </c>
       <c r="I577" t="s">
-        <v>2034</v>
+        <v>2062</v>
       </c>
       <c r="J577" t="s">
         <v>2142</v>
@@ -32917,19 +32917,25 @@
         <v>1337</v>
       </c>
       <c r="C578" t="s">
-        <v>1814</v>
+        <v>1666</v>
+      </c>
+      <c r="D578" t="s">
+        <v>1865</v>
+      </c>
+      <c r="E578" t="s">
+        <v>1905</v>
       </c>
       <c r="F578" s="2">
-        <v>45811</v>
+        <v>45734</v>
       </c>
       <c r="G578" t="s">
-        <v>1918</v>
+        <v>1919</v>
       </c>
       <c r="H578" t="s">
-        <v>1924</v>
+        <v>1950</v>
       </c>
       <c r="I578" t="s">
-        <v>2062</v>
+        <v>2070</v>
       </c>
       <c r="J578" t="s">
         <v>2142</v>
@@ -32949,25 +32955,25 @@
         <v>1338</v>
       </c>
       <c r="C579" t="s">
-        <v>1666</v>
+        <v>1623</v>
       </c>
       <c r="D579" t="s">
-        <v>1865</v>
+        <v>1892</v>
       </c>
       <c r="E579" t="s">
-        <v>1905</v>
+        <v>1904</v>
       </c>
       <c r="F579" s="2">
-        <v>45734</v>
+        <v>45838</v>
       </c>
       <c r="G579" t="s">
-        <v>1919</v>
+        <v>1916</v>
       </c>
       <c r="H579" t="s">
-        <v>1950</v>
+        <v>1933</v>
       </c>
       <c r="I579" t="s">
-        <v>2070</v>
+        <v>2127</v>
       </c>
       <c r="J579" t="s">
         <v>2142</v>
@@ -32987,28 +32993,22 @@
         <v>1339</v>
       </c>
       <c r="C580" t="s">
-        <v>1623</v>
-      </c>
-      <c r="D580" t="s">
-        <v>1892</v>
-      </c>
-      <c r="E580" t="s">
-        <v>1904</v>
+        <v>1815</v>
       </c>
       <c r="F580" s="2">
-        <v>45838</v>
+        <v>45684</v>
       </c>
       <c r="G580" t="s">
         <v>1916</v>
       </c>
       <c r="H580" t="s">
-        <v>1933</v>
+        <v>1920</v>
       </c>
       <c r="I580" t="s">
-        <v>2128</v>
+        <v>2021</v>
       </c>
       <c r="J580" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K580" t="s">
         <v>2719</v>
@@ -33025,22 +33025,22 @@
         <v>1340</v>
       </c>
       <c r="C581" t="s">
-        <v>1815</v>
+        <v>1816</v>
       </c>
       <c r="F581" s="2">
-        <v>45684</v>
+        <v>46092</v>
       </c>
       <c r="G581" t="s">
         <v>1916</v>
       </c>
       <c r="H581" t="s">
-        <v>1920</v>
+        <v>1923</v>
       </c>
       <c r="I581" t="s">
-        <v>2021</v>
+        <v>2037</v>
       </c>
       <c r="J581" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K581" t="s">
         <v>2720</v>
@@ -33057,22 +33057,28 @@
         <v>1341</v>
       </c>
       <c r="C582" t="s">
-        <v>1816</v>
+        <v>1817</v>
+      </c>
+      <c r="D582" t="s">
+        <v>1893</v>
+      </c>
+      <c r="E582" t="s">
+        <v>1562</v>
       </c>
       <c r="F582" s="2">
-        <v>46092</v>
+        <v>45693</v>
       </c>
       <c r="G582" t="s">
         <v>1916</v>
       </c>
       <c r="H582" t="s">
-        <v>1923</v>
+        <v>1924</v>
       </c>
       <c r="I582" t="s">
-        <v>2037</v>
+        <v>1996</v>
       </c>
       <c r="J582" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K582" t="s">
         <v>2721</v>
@@ -33089,16 +33095,10 @@
         <v>1342</v>
       </c>
       <c r="C583" t="s">
-        <v>1817</v>
-      </c>
-      <c r="D583" t="s">
-        <v>1893</v>
-      </c>
-      <c r="E583" t="s">
-        <v>1562</v>
+        <v>1707</v>
       </c>
       <c r="F583" s="2">
-        <v>45693</v>
+        <v>45994</v>
       </c>
       <c r="G583" t="s">
         <v>1916</v>
@@ -33107,10 +33107,10 @@
         <v>1924</v>
       </c>
       <c r="I583" t="s">
-        <v>1996</v>
+        <v>2057</v>
       </c>
       <c r="J583" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K583" t="s">
         <v>2722</v>
@@ -33127,22 +33127,28 @@
         <v>1343</v>
       </c>
       <c r="C584" t="s">
-        <v>1707</v>
+        <v>1648</v>
+      </c>
+      <c r="D584" t="s">
+        <v>1641</v>
+      </c>
+      <c r="E584" t="s">
+        <v>1551</v>
       </c>
       <c r="F584" s="2">
-        <v>45994</v>
+        <v>45923</v>
       </c>
       <c r="G584" t="s">
         <v>1916</v>
       </c>
       <c r="H584" t="s">
-        <v>1924</v>
+        <v>1971</v>
       </c>
       <c r="I584" t="s">
-        <v>2057</v>
+        <v>2128</v>
       </c>
       <c r="J584" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K584" t="s">
         <v>2723</v>
@@ -33159,28 +33165,22 @@
         <v>1344</v>
       </c>
       <c r="C585" t="s">
-        <v>1648</v>
-      </c>
-      <c r="D585" t="s">
-        <v>1641</v>
-      </c>
-      <c r="E585" t="s">
-        <v>1551</v>
+        <v>1818</v>
       </c>
       <c r="F585" s="2">
-        <v>45923</v>
+        <v>46216</v>
       </c>
       <c r="G585" t="s">
         <v>1916</v>
       </c>
       <c r="H585" t="s">
-        <v>1971</v>
+        <v>1936</v>
       </c>
       <c r="I585" t="s">
-        <v>2120</v>
+        <v>2022</v>
       </c>
       <c r="J585" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K585" t="s">
         <v>2724</v>
@@ -33197,19 +33197,19 @@
         <v>1345</v>
       </c>
       <c r="C586" t="s">
-        <v>1818</v>
+        <v>1632</v>
       </c>
       <c r="F586" s="2">
-        <v>46216</v>
+        <v>45712</v>
       </c>
       <c r="G586" t="s">
         <v>1916</v>
       </c>
       <c r="H586" t="s">
-        <v>1936</v>
+        <v>1921</v>
       </c>
       <c r="I586" t="s">
-        <v>2022</v>
+        <v>2016</v>
       </c>
       <c r="J586" t="s">
         <v>2142</v>
@@ -33229,19 +33229,25 @@
         <v>1346</v>
       </c>
       <c r="C587" t="s">
-        <v>1632</v>
+        <v>1544</v>
+      </c>
+      <c r="D587" t="s">
+        <v>1806</v>
+      </c>
+      <c r="E587" t="s">
+        <v>1702</v>
       </c>
       <c r="F587" s="2">
-        <v>45712</v>
+        <v>45848</v>
       </c>
       <c r="G587" t="s">
         <v>1916</v>
       </c>
       <c r="H587" t="s">
-        <v>1921</v>
+        <v>1930</v>
       </c>
       <c r="I587" t="s">
-        <v>2016</v>
+        <v>2004</v>
       </c>
       <c r="J587" t="s">
         <v>2142</v>
@@ -33261,28 +33267,22 @@
         <v>1347</v>
       </c>
       <c r="C588" t="s">
-        <v>1544</v>
-      </c>
-      <c r="D588" t="s">
-        <v>1806</v>
-      </c>
-      <c r="E588" t="s">
-        <v>1702</v>
+        <v>1814</v>
       </c>
       <c r="F588" s="2">
-        <v>45848</v>
+        <v>45722</v>
       </c>
       <c r="G588" t="s">
-        <v>1916</v>
+        <v>1918</v>
       </c>
       <c r="H588" t="s">
-        <v>1930</v>
+        <v>1924</v>
       </c>
       <c r="I588" t="s">
-        <v>2004</v>
+        <v>2129</v>
       </c>
       <c r="J588" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K588" t="s">
         <v>2727</v>
@@ -33299,22 +33299,22 @@
         <v>1348</v>
       </c>
       <c r="C589" t="s">
-        <v>1814</v>
+        <v>1819</v>
       </c>
       <c r="F589" s="2">
-        <v>45722</v>
+        <v>46204</v>
       </c>
       <c r="G589" t="s">
-        <v>1918</v>
+        <v>1916</v>
       </c>
       <c r="H589" t="s">
-        <v>1924</v>
+        <v>1923</v>
       </c>
       <c r="I589" t="s">
-        <v>2129</v>
+        <v>2002</v>
       </c>
       <c r="J589" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K589" t="s">
         <v>2728</v>
@@ -33331,10 +33331,10 @@
         <v>1349</v>
       </c>
       <c r="C590" t="s">
-        <v>1819</v>
+        <v>1694</v>
       </c>
       <c r="F590" s="2">
-        <v>46204</v>
+        <v>45891</v>
       </c>
       <c r="G590" t="s">
         <v>1916</v>
@@ -33343,7 +33343,7 @@
         <v>1923</v>
       </c>
       <c r="I590" t="s">
-        <v>2002</v>
+        <v>2011</v>
       </c>
       <c r="J590" t="s">
         <v>2142</v>
@@ -33363,19 +33363,19 @@
         <v>1350</v>
       </c>
       <c r="C591" t="s">
-        <v>1694</v>
+        <v>1544</v>
       </c>
       <c r="F591" s="2">
-        <v>45891</v>
+        <v>45846</v>
       </c>
       <c r="G591" t="s">
         <v>1916</v>
       </c>
       <c r="H591" t="s">
-        <v>1923</v>
+        <v>1926</v>
       </c>
       <c r="I591" t="s">
-        <v>2011</v>
+        <v>2004</v>
       </c>
       <c r="J591" t="s">
         <v>2142</v>
@@ -33395,7 +33395,7 @@
         <v>1351</v>
       </c>
       <c r="C592" t="s">
-        <v>1544</v>
+        <v>1643</v>
       </c>
       <c r="F592" s="2">
         <v>45846</v>
@@ -33404,10 +33404,10 @@
         <v>1916</v>
       </c>
       <c r="H592" t="s">
-        <v>1926</v>
+        <v>1921</v>
       </c>
       <c r="I592" t="s">
-        <v>2004</v>
+        <v>1982</v>
       </c>
       <c r="J592" t="s">
         <v>2142</v>
@@ -33427,19 +33427,19 @@
         <v>1352</v>
       </c>
       <c r="C593" t="s">
-        <v>1643</v>
+        <v>1608</v>
       </c>
       <c r="F593" s="2">
-        <v>45846</v>
+        <v>46175</v>
       </c>
       <c r="G593" t="s">
         <v>1916</v>
       </c>
       <c r="H593" t="s">
-        <v>1921</v>
+        <v>1926</v>
       </c>
       <c r="I593" t="s">
-        <v>1982</v>
+        <v>2130</v>
       </c>
       <c r="J593" t="s">
         <v>2142</v>
@@ -33459,19 +33459,19 @@
         <v>1353</v>
       </c>
       <c r="C594" t="s">
-        <v>1608</v>
+        <v>1782</v>
       </c>
       <c r="F594" s="2">
-        <v>46175</v>
+        <v>45994</v>
       </c>
       <c r="G594" t="s">
         <v>1916</v>
       </c>
       <c r="H594" t="s">
-        <v>1926</v>
+        <v>1924</v>
       </c>
       <c r="I594" t="s">
-        <v>2130</v>
+        <v>2013</v>
       </c>
       <c r="J594" t="s">
         <v>2142</v>
@@ -33491,19 +33491,22 @@
         <v>1354</v>
       </c>
       <c r="C595" t="s">
-        <v>1782</v>
+        <v>1820</v>
+      </c>
+      <c r="D595" t="s">
+        <v>1553</v>
       </c>
       <c r="F595" s="2">
-        <v>45994</v>
+        <v>45946</v>
       </c>
       <c r="G595" t="s">
         <v>1916</v>
       </c>
       <c r="H595" t="s">
-        <v>1924</v>
+        <v>1943</v>
       </c>
       <c r="I595" t="s">
-        <v>2013</v>
+        <v>2131</v>
       </c>
       <c r="J595" t="s">
         <v>2142</v>
@@ -33523,13 +33526,13 @@
         <v>1355</v>
       </c>
       <c r="C596" t="s">
-        <v>1820</v>
+        <v>1548</v>
       </c>
       <c r="D596" t="s">
-        <v>1553</v>
+        <v>1714</v>
       </c>
       <c r="F596" s="2">
-        <v>45946</v>
+        <v>46162</v>
       </c>
       <c r="G596" t="s">
         <v>1916</v>
@@ -33538,10 +33541,10 @@
         <v>1943</v>
       </c>
       <c r="I596" t="s">
-        <v>2131</v>
+        <v>2010</v>
       </c>
       <c r="J596" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K596" t="s">
         <v>2735</v>
@@ -33558,25 +33561,28 @@
         <v>1356</v>
       </c>
       <c r="C597" t="s">
-        <v>1548</v>
+        <v>1821</v>
       </c>
       <c r="D597" t="s">
-        <v>1714</v>
+        <v>1703</v>
+      </c>
+      <c r="E597" t="s">
+        <v>1703</v>
       </c>
       <c r="F597" s="2">
-        <v>46162</v>
+        <v>45950</v>
       </c>
       <c r="G597" t="s">
         <v>1916</v>
       </c>
       <c r="H597" t="s">
-        <v>1943</v>
+        <v>1933</v>
       </c>
       <c r="I597" t="s">
-        <v>2010</v>
+        <v>1978</v>
       </c>
       <c r="J597" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K597" t="s">
         <v>2736</v>
@@ -33593,25 +33599,19 @@
         <v>1357</v>
       </c>
       <c r="C598" t="s">
-        <v>1821</v>
-      </c>
-      <c r="D598" t="s">
-        <v>1703</v>
-      </c>
-      <c r="E598" t="s">
-        <v>1703</v>
+        <v>1822</v>
       </c>
       <c r="F598" s="2">
-        <v>45950</v>
+        <v>45679</v>
       </c>
       <c r="G598" t="s">
-        <v>1916</v>
+        <v>1919</v>
       </c>
       <c r="H598" t="s">
-        <v>1933</v>
+        <v>1926</v>
       </c>
       <c r="I598" t="s">
-        <v>1978</v>
+        <v>1976</v>
       </c>
       <c r="J598" t="s">
         <v>2142</v>
@@ -33631,19 +33631,25 @@
         <v>1358</v>
       </c>
       <c r="C599" t="s">
-        <v>1822</v>
+        <v>1664</v>
+      </c>
+      <c r="D599" t="s">
+        <v>1775</v>
+      </c>
+      <c r="E599" t="s">
+        <v>1826</v>
       </c>
       <c r="F599" s="2">
-        <v>45679</v>
+        <v>45915</v>
       </c>
       <c r="G599" t="s">
-        <v>1919</v>
+        <v>1916</v>
       </c>
       <c r="H599" t="s">
-        <v>1926</v>
+        <v>1955</v>
       </c>
       <c r="I599" t="s">
-        <v>1976</v>
+        <v>2051</v>
       </c>
       <c r="J599" t="s">
         <v>2142</v>
@@ -33663,25 +33669,19 @@
         <v>1359</v>
       </c>
       <c r="C600" t="s">
-        <v>1664</v>
-      </c>
-      <c r="D600" t="s">
-        <v>1775</v>
-      </c>
-      <c r="E600" t="s">
-        <v>1826</v>
+        <v>1588</v>
       </c>
       <c r="F600" s="2">
-        <v>45915</v>
+        <v>45754</v>
       </c>
       <c r="G600" t="s">
-        <v>1916</v>
+        <v>1918</v>
       </c>
       <c r="H600" t="s">
-        <v>1955</v>
+        <v>1924</v>
       </c>
       <c r="I600" t="s">
-        <v>2051</v>
+        <v>2011</v>
       </c>
       <c r="J600" t="s">
         <v>2142</v>
@@ -33701,19 +33701,19 @@
         <v>1360</v>
       </c>
       <c r="C601" t="s">
-        <v>1588</v>
+        <v>1732</v>
       </c>
       <c r="F601" s="2">
-        <v>45754</v>
+        <v>45835</v>
       </c>
       <c r="G601" t="s">
-        <v>1918</v>
+        <v>1916</v>
       </c>
       <c r="H601" t="s">
-        <v>1924</v>
+        <v>1926</v>
       </c>
       <c r="I601" t="s">
-        <v>2011</v>
+        <v>1987</v>
       </c>
       <c r="J601" t="s">
         <v>2142</v>
@@ -33733,19 +33733,19 @@
         <v>1361</v>
       </c>
       <c r="C602" t="s">
-        <v>1732</v>
+        <v>1514</v>
       </c>
       <c r="F602" s="2">
-        <v>45835</v>
+        <v>45751</v>
       </c>
       <c r="G602" t="s">
         <v>1916</v>
       </c>
       <c r="H602" t="s">
-        <v>1926</v>
+        <v>1972</v>
       </c>
       <c r="I602" t="s">
-        <v>1987</v>
+        <v>2109</v>
       </c>
       <c r="J602" t="s">
         <v>2142</v>
@@ -33765,19 +33765,25 @@
         <v>1362</v>
       </c>
       <c r="C603" t="s">
-        <v>1514</v>
+        <v>1607</v>
+      </c>
+      <c r="D603" t="s">
+        <v>1627</v>
+      </c>
+      <c r="E603" t="s">
+        <v>1511</v>
       </c>
       <c r="F603" s="2">
-        <v>45751</v>
+        <v>46219</v>
       </c>
       <c r="G603" t="s">
         <v>1916</v>
       </c>
       <c r="H603" t="s">
-        <v>1972</v>
+        <v>1933</v>
       </c>
       <c r="I603" t="s">
-        <v>2109</v>
+        <v>1997</v>
       </c>
       <c r="J603" t="s">
         <v>2142</v>
@@ -33797,25 +33803,19 @@
         <v>1363</v>
       </c>
       <c r="C604" t="s">
-        <v>1607</v>
-      </c>
-      <c r="D604" t="s">
-        <v>1627</v>
-      </c>
-      <c r="E604" t="s">
-        <v>1511</v>
+        <v>1732</v>
       </c>
       <c r="F604" s="2">
-        <v>46219</v>
+        <v>45853</v>
       </c>
       <c r="G604" t="s">
         <v>1916</v>
       </c>
       <c r="H604" t="s">
-        <v>1933</v>
+        <v>1946</v>
       </c>
       <c r="I604" t="s">
-        <v>1997</v>
+        <v>2076</v>
       </c>
       <c r="J604" t="s">
         <v>2142</v>
@@ -33835,19 +33835,19 @@
         <v>1364</v>
       </c>
       <c r="C605" t="s">
-        <v>1732</v>
+        <v>1743</v>
       </c>
       <c r="F605" s="2">
-        <v>45853</v>
+        <v>46196</v>
       </c>
       <c r="G605" t="s">
         <v>1916</v>
       </c>
       <c r="H605" t="s">
-        <v>1946</v>
+        <v>1923</v>
       </c>
       <c r="I605" t="s">
-        <v>2076</v>
+        <v>2009</v>
       </c>
       <c r="J605" t="s">
         <v>2142</v>
@@ -33867,19 +33867,19 @@
         <v>1365</v>
       </c>
       <c r="C606" t="s">
-        <v>1743</v>
+        <v>1637</v>
       </c>
       <c r="F606" s="2">
-        <v>46196</v>
+        <v>45911</v>
       </c>
       <c r="G606" t="s">
         <v>1916</v>
       </c>
       <c r="H606" t="s">
-        <v>1923</v>
+        <v>1943</v>
       </c>
       <c r="I606" t="s">
-        <v>2009</v>
+        <v>2020</v>
       </c>
       <c r="J606" t="s">
         <v>2142</v>
@@ -33899,19 +33899,25 @@
         <v>1366</v>
       </c>
       <c r="C607" t="s">
-        <v>1637</v>
+        <v>1687</v>
+      </c>
+      <c r="D607" t="s">
+        <v>1576</v>
+      </c>
+      <c r="E607" t="s">
+        <v>1576</v>
       </c>
       <c r="F607" s="2">
-        <v>45911</v>
+        <v>45996</v>
       </c>
       <c r="G607" t="s">
         <v>1916</v>
       </c>
       <c r="H607" t="s">
-        <v>1943</v>
+        <v>1938</v>
       </c>
       <c r="I607" t="s">
-        <v>2020</v>
+        <v>1987</v>
       </c>
       <c r="J607" t="s">
         <v>2142</v>
@@ -33931,25 +33937,19 @@
         <v>1367</v>
       </c>
       <c r="C608" t="s">
-        <v>1687</v>
-      </c>
-      <c r="D608" t="s">
-        <v>1576</v>
-      </c>
-      <c r="E608" t="s">
-        <v>1576</v>
+        <v>1714</v>
       </c>
       <c r="F608" s="2">
-        <v>45996</v>
+        <v>46003</v>
       </c>
       <c r="G608" t="s">
         <v>1916</v>
       </c>
       <c r="H608" t="s">
-        <v>1938</v>
+        <v>1921</v>
       </c>
       <c r="I608" t="s">
-        <v>1987</v>
+        <v>2053</v>
       </c>
       <c r="J608" t="s">
         <v>2142</v>
@@ -33969,19 +33969,25 @@
         <v>1368</v>
       </c>
       <c r="C609" t="s">
-        <v>1714</v>
+        <v>1735</v>
+      </c>
+      <c r="D609" t="s">
+        <v>1669</v>
+      </c>
+      <c r="E609" t="s">
+        <v>1669</v>
       </c>
       <c r="F609" s="2">
-        <v>46003</v>
+        <v>45937</v>
       </c>
       <c r="G609" t="s">
         <v>1916</v>
       </c>
       <c r="H609" t="s">
-        <v>1921</v>
+        <v>1956</v>
       </c>
       <c r="I609" t="s">
-        <v>2053</v>
+        <v>1987</v>
       </c>
       <c r="J609" t="s">
         <v>2142</v>
@@ -34001,25 +34007,19 @@
         <v>1369</v>
       </c>
       <c r="C610" t="s">
-        <v>1735</v>
-      </c>
-      <c r="D610" t="s">
-        <v>1669</v>
-      </c>
-      <c r="E610" t="s">
-        <v>1669</v>
+        <v>1744</v>
       </c>
       <c r="F610" s="2">
-        <v>45937</v>
+        <v>46204</v>
       </c>
       <c r="G610" t="s">
         <v>1916</v>
       </c>
       <c r="H610" t="s">
-        <v>1956</v>
+        <v>1924</v>
       </c>
       <c r="I610" t="s">
-        <v>1987</v>
+        <v>2002</v>
       </c>
       <c r="J610" t="s">
         <v>2142</v>
@@ -34039,19 +34039,19 @@
         <v>1370</v>
       </c>
       <c r="C611" t="s">
-        <v>1744</v>
+        <v>1729</v>
       </c>
       <c r="F611" s="2">
-        <v>46204</v>
+        <v>46168</v>
       </c>
       <c r="G611" t="s">
         <v>1916</v>
       </c>
       <c r="H611" t="s">
-        <v>1924</v>
+        <v>1936</v>
       </c>
       <c r="I611" t="s">
-        <v>2002</v>
+        <v>1980</v>
       </c>
       <c r="J611" t="s">
         <v>2142</v>
@@ -34071,19 +34071,19 @@
         <v>1371</v>
       </c>
       <c r="C612" t="s">
-        <v>1729</v>
+        <v>1823</v>
       </c>
       <c r="F612" s="2">
-        <v>46168</v>
+        <v>45824</v>
       </c>
       <c r="G612" t="s">
         <v>1916</v>
       </c>
       <c r="H612" t="s">
-        <v>1936</v>
+        <v>1926</v>
       </c>
       <c r="I612" t="s">
-        <v>1980</v>
+        <v>2132</v>
       </c>
       <c r="J612" t="s">
         <v>2142</v>
@@ -34103,19 +34103,22 @@
         <v>1372</v>
       </c>
       <c r="C613" t="s">
-        <v>1823</v>
+        <v>1659</v>
+      </c>
+      <c r="D613" t="s">
+        <v>1894</v>
       </c>
       <c r="F613" s="2">
-        <v>45824</v>
+        <v>46050</v>
       </c>
       <c r="G613" t="s">
         <v>1916</v>
       </c>
       <c r="H613" t="s">
-        <v>1926</v>
+        <v>1921</v>
       </c>
       <c r="I613" t="s">
-        <v>2132</v>
+        <v>2035</v>
       </c>
       <c r="J613" t="s">
         <v>2142</v>
@@ -34135,22 +34138,19 @@
         <v>1373</v>
       </c>
       <c r="C614" t="s">
-        <v>1659</v>
-      </c>
-      <c r="D614" t="s">
-        <v>1894</v>
+        <v>1642</v>
       </c>
       <c r="F614" s="2">
-        <v>46050</v>
+        <v>45908</v>
       </c>
       <c r="G614" t="s">
         <v>1916</v>
       </c>
       <c r="H614" t="s">
-        <v>1921</v>
+        <v>1924</v>
       </c>
       <c r="I614" t="s">
-        <v>2035</v>
+        <v>1976</v>
       </c>
       <c r="J614" t="s">
         <v>2142</v>
@@ -34170,19 +34170,19 @@
         <v>1374</v>
       </c>
       <c r="C615" t="s">
-        <v>1642</v>
+        <v>1538</v>
       </c>
       <c r="F615" s="2">
-        <v>45908</v>
+        <v>46175</v>
       </c>
       <c r="G615" t="s">
         <v>1916</v>
       </c>
       <c r="H615" t="s">
-        <v>1924</v>
+        <v>1965</v>
       </c>
       <c r="I615" t="s">
-        <v>1976</v>
+        <v>1979</v>
       </c>
       <c r="J615" t="s">
         <v>2142</v>
@@ -34202,22 +34202,28 @@
         <v>1375</v>
       </c>
       <c r="C616" t="s">
-        <v>1538</v>
+        <v>1511</v>
+      </c>
+      <c r="D616" t="s">
+        <v>1895</v>
+      </c>
+      <c r="E616" t="s">
+        <v>1895</v>
       </c>
       <c r="F616" s="2">
-        <v>46175</v>
+        <v>46217</v>
       </c>
       <c r="G616" t="s">
         <v>1916</v>
       </c>
       <c r="H616" t="s">
-        <v>1965</v>
+        <v>1938</v>
       </c>
       <c r="I616" t="s">
-        <v>1979</v>
+        <v>1987</v>
       </c>
       <c r="J616" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K616" t="s">
         <v>2755</v>
@@ -34234,28 +34240,22 @@
         <v>1376</v>
       </c>
       <c r="C617" t="s">
-        <v>1511</v>
-      </c>
-      <c r="D617" t="s">
-        <v>1895</v>
-      </c>
-      <c r="E617" t="s">
-        <v>1895</v>
+        <v>1782</v>
       </c>
       <c r="F617" s="2">
-        <v>46217</v>
+        <v>46093</v>
       </c>
       <c r="G617" t="s">
         <v>1916</v>
       </c>
       <c r="H617" t="s">
-        <v>1938</v>
+        <v>1923</v>
       </c>
       <c r="I617" t="s">
-        <v>1987</v>
+        <v>2034</v>
       </c>
       <c r="J617" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K617" t="s">
         <v>2756</v>
@@ -34272,22 +34272,28 @@
         <v>1377</v>
       </c>
       <c r="C618" t="s">
-        <v>1782</v>
+        <v>1777</v>
+      </c>
+      <c r="D618" t="s">
+        <v>1693</v>
+      </c>
+      <c r="E618" t="s">
+        <v>1766</v>
       </c>
       <c r="F618" s="2">
-        <v>46093</v>
+        <v>45750</v>
       </c>
       <c r="G618" t="s">
         <v>1916</v>
       </c>
       <c r="H618" t="s">
-        <v>1923</v>
+        <v>1932</v>
       </c>
       <c r="I618" t="s">
-        <v>2034</v>
+        <v>2128</v>
       </c>
       <c r="J618" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K618" t="s">
         <v>2757</v>
@@ -34304,28 +34310,22 @@
         <v>1378</v>
       </c>
       <c r="C619" t="s">
-        <v>1777</v>
-      </c>
-      <c r="D619" t="s">
-        <v>1693</v>
-      </c>
-      <c r="E619" t="s">
-        <v>1766</v>
+        <v>1824</v>
       </c>
       <c r="F619" s="2">
-        <v>45750</v>
+        <v>45946</v>
       </c>
       <c r="G619" t="s">
-        <v>1916</v>
+        <v>1917</v>
       </c>
       <c r="H619" t="s">
-        <v>1932</v>
+        <v>1926</v>
       </c>
       <c r="I619" t="s">
-        <v>2120</v>
+        <v>1980</v>
       </c>
       <c r="J619" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K619" t="s">
         <v>2758</v>
@@ -34342,19 +34342,19 @@
         <v>1379</v>
       </c>
       <c r="C620" t="s">
-        <v>1824</v>
+        <v>1825</v>
       </c>
       <c r="F620" s="2">
-        <v>45946</v>
+        <v>45751</v>
       </c>
       <c r="G620" t="s">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="H620" t="s">
-        <v>1926</v>
+        <v>1923</v>
       </c>
       <c r="I620" t="s">
-        <v>1980</v>
+        <v>2043</v>
       </c>
       <c r="J620" t="s">
         <v>2142</v>
@@ -34374,22 +34374,28 @@
         <v>1380</v>
       </c>
       <c r="C621" t="s">
-        <v>1825</v>
+        <v>1692</v>
+      </c>
+      <c r="D621" t="s">
+        <v>1896</v>
+      </c>
+      <c r="E621" t="s">
+        <v>1863</v>
       </c>
       <c r="F621" s="2">
-        <v>45751</v>
+        <v>46176</v>
       </c>
       <c r="G621" t="s">
-        <v>1916</v>
+        <v>1918</v>
       </c>
       <c r="H621" t="s">
         <v>1923</v>
       </c>
       <c r="I621" t="s">
-        <v>2043</v>
+        <v>2129</v>
       </c>
       <c r="J621" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K621" t="s">
         <v>2760</v>
@@ -34406,28 +34412,22 @@
         <v>1381</v>
       </c>
       <c r="C622" t="s">
-        <v>1692</v>
-      </c>
-      <c r="D622" t="s">
-        <v>1896</v>
-      </c>
-      <c r="E622" t="s">
-        <v>1863</v>
+        <v>1697</v>
       </c>
       <c r="F622" s="2">
-        <v>46176</v>
+        <v>45938</v>
       </c>
       <c r="G622" t="s">
-        <v>1918</v>
+        <v>1916</v>
       </c>
       <c r="H622" t="s">
         <v>1923</v>
       </c>
       <c r="I622" t="s">
-        <v>2129</v>
+        <v>1980</v>
       </c>
       <c r="J622" t="s">
-        <v>2143</v>
+        <v>2142</v>
       </c>
       <c r="K622" t="s">
         <v>2761</v>
@@ -34444,19 +34444,19 @@
         <v>1382</v>
       </c>
       <c r="C623" t="s">
-        <v>1697</v>
+        <v>1556</v>
       </c>
       <c r="F623" s="2">
-        <v>45938</v>
+        <v>46118</v>
       </c>
       <c r="G623" t="s">
         <v>1916</v>
       </c>
       <c r="H623" t="s">
-        <v>1923</v>
+        <v>1926</v>
       </c>
       <c r="I623" t="s">
-        <v>1980</v>
+        <v>2019</v>
       </c>
       <c r="J623" t="s">
         <v>2142</v>
@@ -34476,19 +34476,19 @@
         <v>1383</v>
       </c>
       <c r="C624" t="s">
-        <v>1556</v>
+        <v>1748</v>
       </c>
       <c r="F624" s="2">
-        <v>46118</v>
+        <v>45994</v>
       </c>
       <c r="G624" t="s">
         <v>1916</v>
       </c>
       <c r="H624" t="s">
-        <v>1926</v>
+        <v>1923</v>
       </c>
       <c r="I624" t="s">
-        <v>2019</v>
+        <v>2034</v>
       </c>
       <c r="J624" t="s">
         <v>2142</v>
@@ -34508,19 +34508,25 @@
         <v>1384</v>
       </c>
       <c r="C625" t="s">
-        <v>1748</v>
+        <v>1680</v>
+      </c>
+      <c r="D625" t="s">
+        <v>1605</v>
+      </c>
+      <c r="E625" t="s">
+        <v>1524</v>
       </c>
       <c r="F625" s="2">
-        <v>45994</v>
+        <v>45859</v>
       </c>
       <c r="G625" t="s">
-        <v>1916</v>
+        <v>1917</v>
       </c>
       <c r="H625" t="s">
-        <v>1923</v>
+        <v>1921</v>
       </c>
       <c r="I625" t="s">
-        <v>2034</v>
+        <v>1980</v>
       </c>
       <c r="J625" t="s">
         <v>2142</v>
@@ -34540,25 +34546,19 @@
         <v>1385</v>
       </c>
       <c r="C626" t="s">
-        <v>1680</v>
-      </c>
-      <c r="D626" t="s">
-        <v>1605</v>
-      </c>
-      <c r="E626" t="s">
-        <v>1524</v>
+        <v>1826</v>
       </c>
       <c r="F626" s="2">
-        <v>45859</v>
+        <v>46049</v>
       </c>
       <c r="G626" t="s">
-        <v>1917</v>
+        <v>1916</v>
       </c>
       <c r="H626" t="s">
-        <v>1921</v>
+        <v>1923</v>
       </c>
       <c r="I626" t="s">
-        <v>1980</v>
+        <v>1976</v>
       </c>
       <c r="J626" t="s">
         <v>2142</v>
@@ -34578,19 +34578,19 @@
         <v>1386</v>
       </c>
       <c r="C627" t="s">
-        <v>1826</v>
+        <v>1739</v>
       </c>
       <c r="F627" s="2">
-        <v>46049</v>
+        <v>46118</v>
       </c>
       <c r="G627" t="s">
         <v>1916</v>
       </c>
       <c r="H627" t="s">
-        <v>1923</v>
+        <v>1926</v>
       </c>
       <c r="I627" t="s">
-        <v>1976</v>
+        <v>2029</v>
       </c>
       <c r="J627" t="s">
         <v>2142</v>
@@ -34610,22 +34610,22 @@
         <v>1387</v>
       </c>
       <c r="C628" t="s">
-        <v>1739</v>
+        <v>1578</v>
       </c>
       <c r="F628" s="2">
-        <v>46118</v>
+        <v>45923</v>
       </c>
       <c r="G628" t="s">
         <v>1916</v>
       </c>
       <c r="H628" t="s">
-        <v>1926</v>
+        <v>1925</v>
       </c>
       <c r="I628" t="s">
-        <v>2029</v>
+        <v>2057</v>
       </c>
       <c r="J628" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="K628" t="s">
         <v>2767</v>
@@ -34642,19 +34642,25 @@
         <v>1388</v>
       </c>
       <c r="C629" t="s">
-        <v>1578</v>
+        <v>1808</v>
+      </c>
+      <c r="D629" t="s">
+        <v>1889</v>
+      </c>
+      <c r="E629" t="s">
+        <v>1889</v>
       </c>
       <c r="F629" s="2">
-        <v>45923</v>
+        <v>46234</v>
       </c>
       <c r="G629" t="s">
-        <v>1916</v>
+        <v>1917</v>
       </c>
       <c r="H629" t="s">
-        <v>1925</v>
+        <v>1961</v>
       </c>
       <c r="I629" t="s">
-        <v>2057</v>
+        <v>2051</v>
       </c>
       <c r="J629" t="s">
         <v>2143</v>
@@ -34750,7 +34756,7 @@
         <v>1926</v>
       </c>
       <c r="I632" t="s">
-        <v>2124</v>
+        <v>2123</v>
       </c>
       <c r="J632" t="s">
         <v>2143</v>
@@ -36216,7 +36222,7 @@
         <v>1925</v>
       </c>
       <c r="I675" t="s">
-        <v>2120</v>
+        <v>2128</v>
       </c>
       <c r="J675" t="s">
         <v>2143</v>
@@ -36248,7 +36254,7 @@
         <v>1975</v>
       </c>
       <c r="I676" t="s">
-        <v>2123</v>
+        <v>2122</v>
       </c>
       <c r="J676" t="s">
         <v>2142</v>

</xml_diff>